<commit_message>
POS test case added
</commit_message>
<xml_diff>
--- a/src/main/resources/ClientPortal_Data.xlsx
+++ b/src/main/resources/ClientPortal_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BS01361\My Folder\0. Test Type\4. Automation Testing\Selenium Files\MAS_FloraFire\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB0F3F6E-0BFC-4A14-9A56-B89841F4F3AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1BFD2C-D3FA-4774-B731-DCC354703090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="803" firstSheet="1" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="803" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Value" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
     <sheet name="ShortCuts" sheetId="6" r:id="rId15"/>
     <sheet name="Test" sheetId="22" r:id="rId16"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2132,19 +2132,19 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3947,7 +3947,7 @@
       <c r="D2" s="8">
         <v>1</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="25" t="s">
         <v>81</v>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       <c r="D3" s="2">
         <v>0</v>
       </c>
-      <c r="E3" s="28"/>
+      <c r="E3" s="29"/>
     </row>
     <row r="4" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
@@ -3979,7 +3979,7 @@
       <c r="D4" s="11">
         <v>-1</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="26"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -3994,7 +3994,7 @@
       <c r="D5" s="8">
         <v>1</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="25" t="s">
         <v>82</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -4014,7 +4014,7 @@
       <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6" s="28"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
@@ -4029,7 +4029,7 @@
       <c r="D7" s="6">
         <v>-1</v>
       </c>
-      <c r="E7" s="29"/>
+      <c r="E7" s="26"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -4044,7 +4044,7 @@
       <c r="D8" s="8">
         <v>1</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="25" t="s">
         <v>83</v>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       <c r="D9" s="2">
         <v>0</v>
       </c>
-      <c r="E9" s="28"/>
+      <c r="E9" s="29"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
@@ -4076,7 +4076,7 @@
       <c r="D10" s="2">
         <v>0</v>
       </c>
-      <c r="E10" s="28"/>
+      <c r="E10" s="29"/>
     </row>
     <row r="11" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
@@ -4091,7 +4091,7 @@
       <c r="D11" s="6">
         <v>-1</v>
       </c>
-      <c r="E11" s="28"/>
+      <c r="E11" s="29"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -4106,7 +4106,7 @@
       <c r="D12" s="8">
         <v>1</v>
       </c>
-      <c r="E12" s="27" t="s">
+      <c r="E12" s="25" t="s">
         <v>68</v>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
       <c r="D13" s="11">
         <v>-1</v>
       </c>
-      <c r="E13" s="29"/>
+      <c r="E13" s="26"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
@@ -4138,7 +4138,7 @@
       <c r="D14" s="8">
         <v>1</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="25" t="s">
         <v>69</v>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="E15" s="28"/>
+      <c r="E15" s="29"/>
     </row>
     <row r="16" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
@@ -4170,7 +4170,7 @@
       <c r="D16" s="6">
         <v>-1</v>
       </c>
-      <c r="E16" s="29"/>
+      <c r="E16" s="26"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
@@ -4185,7 +4185,7 @@
       <c r="D17" s="8">
         <v>1</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="25" t="s">
         <v>70</v>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
       <c r="D18" s="11">
         <v>-1</v>
       </c>
-      <c r="E18" s="29"/>
+      <c r="E18" s="26"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
@@ -4217,7 +4217,7 @@
       <c r="D19" s="8">
         <v>1</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="25" t="s">
         <v>71</v>
       </c>
     </row>
@@ -4234,7 +4234,7 @@
       <c r="D20" s="2">
         <v>0</v>
       </c>
-      <c r="E20" s="28"/>
+      <c r="E20" s="29"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
@@ -4249,7 +4249,7 @@
       <c r="D21" s="2">
         <v>0</v>
       </c>
-      <c r="E21" s="28"/>
+      <c r="E21" s="29"/>
     </row>
     <row r="22" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
@@ -4264,7 +4264,7 @@
       <c r="D22" s="6">
         <v>-1</v>
       </c>
-      <c r="E22" s="29"/>
+      <c r="E22" s="26"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
@@ -4279,7 +4279,7 @@
       <c r="D23" s="8">
         <v>1</v>
       </c>
-      <c r="E23" s="27" t="s">
+      <c r="E23" s="25" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4296,7 +4296,7 @@
       <c r="D24" s="2">
         <v>0</v>
       </c>
-      <c r="E24" s="28"/>
+      <c r="E24" s="29"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
@@ -4311,7 +4311,7 @@
       <c r="D25" s="2">
         <v>0</v>
       </c>
-      <c r="E25" s="28"/>
+      <c r="E25" s="29"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
@@ -4326,7 +4326,7 @@
       <c r="D26" s="2">
         <v>0</v>
       </c>
-      <c r="E26" s="28"/>
+      <c r="E26" s="29"/>
     </row>
     <row r="27" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
@@ -4341,7 +4341,7 @@
       <c r="D27" s="11">
         <v>-1</v>
       </c>
-      <c r="E27" s="29"/>
+      <c r="E27" s="26"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
@@ -4356,7 +4356,7 @@
       <c r="D28" s="8">
         <v>1</v>
       </c>
-      <c r="E28" s="27" t="s">
+      <c r="E28" s="25" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
       <c r="D29" s="2">
         <v>0</v>
       </c>
-      <c r="E29" s="28"/>
+      <c r="E29" s="29"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
@@ -4388,7 +4388,7 @@
       <c r="D30" s="2">
         <v>0</v>
       </c>
-      <c r="E30" s="28"/>
+      <c r="E30" s="29"/>
     </row>
     <row r="31" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
@@ -4403,7 +4403,7 @@
       <c r="D31" s="6">
         <v>-1</v>
       </c>
-      <c r="E31" s="29"/>
+      <c r="E31" s="26"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
@@ -4418,7 +4418,7 @@
       <c r="D32" s="8">
         <v>1</v>
       </c>
-      <c r="E32" s="27" t="s">
+      <c r="E32" s="25" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4435,7 +4435,7 @@
       <c r="D33" s="2">
         <v>0</v>
       </c>
-      <c r="E33" s="28"/>
+      <c r="E33" s="29"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
@@ -4450,7 +4450,7 @@
       <c r="D34" s="2">
         <v>0</v>
       </c>
-      <c r="E34" s="28"/>
+      <c r="E34" s="29"/>
     </row>
     <row r="35" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
@@ -4465,7 +4465,7 @@
       <c r="D35" s="6">
         <v>-1</v>
       </c>
-      <c r="E35" s="29"/>
+      <c r="E35" s="26"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
@@ -4480,7 +4480,7 @@
       <c r="D36" s="8">
         <v>1</v>
       </c>
-      <c r="E36" s="27" t="s">
+      <c r="E36" s="25" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4497,7 +4497,7 @@
       <c r="D37" s="11">
         <v>-1</v>
       </c>
-      <c r="E37" s="29"/>
+      <c r="E37" s="26"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
@@ -4512,7 +4512,7 @@
       <c r="D38" s="8">
         <v>1</v>
       </c>
-      <c r="E38" s="27" t="s">
+      <c r="E38" s="25" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
       <c r="D39" s="11">
         <v>-1</v>
       </c>
-      <c r="E39" s="29"/>
+      <c r="E39" s="26"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
@@ -4544,7 +4544,7 @@
       <c r="D40" s="8">
         <v>1</v>
       </c>
-      <c r="E40" s="27" t="s">
+      <c r="E40" s="25" t="s">
         <v>77</v>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       <c r="D41" s="2">
         <v>0</v>
       </c>
-      <c r="E41" s="28"/>
+      <c r="E41" s="29"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
@@ -4576,7 +4576,7 @@
       <c r="D42" s="2">
         <v>0</v>
       </c>
-      <c r="E42" s="28"/>
+      <c r="E42" s="29"/>
     </row>
     <row r="43" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
@@ -4591,7 +4591,7 @@
       <c r="D43" s="6">
         <v>-1</v>
       </c>
-      <c r="E43" s="29"/>
+      <c r="E43" s="26"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
@@ -4606,7 +4606,7 @@
       <c r="D44" s="8">
         <v>1</v>
       </c>
-      <c r="E44" s="27" t="s">
+      <c r="E44" s="25" t="s">
         <v>78</v>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       <c r="D45" s="2">
         <v>0</v>
       </c>
-      <c r="E45" s="28"/>
+      <c r="E45" s="29"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
@@ -4638,7 +4638,7 @@
       <c r="D46" s="2">
         <v>0</v>
       </c>
-      <c r="E46" s="28"/>
+      <c r="E46" s="29"/>
     </row>
     <row r="47" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
@@ -4653,7 +4653,7 @@
       <c r="D47" s="6">
         <v>-1</v>
       </c>
-      <c r="E47" s="29"/>
+      <c r="E47" s="26"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
@@ -4668,7 +4668,7 @@
       <c r="D48" s="8">
         <v>1</v>
       </c>
-      <c r="E48" s="27" t="s">
+      <c r="E48" s="25" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4685,7 +4685,7 @@
       <c r="D49" s="2">
         <v>0</v>
       </c>
-      <c r="E49" s="28"/>
+      <c r="E49" s="29"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
@@ -4700,7 +4700,7 @@
       <c r="D50" s="2">
         <v>0</v>
       </c>
-      <c r="E50" s="28"/>
+      <c r="E50" s="29"/>
     </row>
     <row r="51" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
@@ -4715,7 +4715,7 @@
       <c r="D51" s="6">
         <v>-1</v>
       </c>
-      <c r="E51" s="29"/>
+      <c r="E51" s="26"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
@@ -4730,7 +4730,7 @@
       <c r="D52" s="8">
         <v>1</v>
       </c>
-      <c r="E52" s="27" t="s">
+      <c r="E52" s="25" t="s">
         <v>80</v>
       </c>
     </row>
@@ -4747,7 +4747,7 @@
       <c r="D53" s="2">
         <v>0</v>
       </c>
-      <c r="E53" s="28"/>
+      <c r="E53" s="29"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
@@ -4762,7 +4762,7 @@
       <c r="D54" s="2">
         <v>0</v>
       </c>
-      <c r="E54" s="28"/>
+      <c r="E54" s="29"/>
     </row>
     <row r="55" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="12" t="s">
@@ -4777,7 +4777,7 @@
       <c r="D55" s="6">
         <v>-1</v>
       </c>
-      <c r="E55" s="28"/>
+      <c r="E55" s="29"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
@@ -4792,7 +4792,7 @@
       <c r="D56" s="8">
         <v>1</v>
       </c>
-      <c r="E56" s="25" t="s">
+      <c r="E56" s="27" t="s">
         <v>498</v>
       </c>
     </row>
@@ -4809,7 +4809,7 @@
       <c r="D57" s="6">
         <v>-1</v>
       </c>
-      <c r="E57" s="26"/>
+      <c r="E57" s="28"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
@@ -4824,7 +4824,7 @@
       <c r="D58" s="8">
         <v>1</v>
       </c>
-      <c r="E58" s="27" t="s">
+      <c r="E58" s="25" t="s">
         <v>499</v>
       </c>
     </row>
@@ -4841,7 +4841,7 @@
       <c r="D59" s="2">
         <v>0</v>
       </c>
-      <c r="E59" s="28"/>
+      <c r="E59" s="29"/>
     </row>
     <row r="60" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
@@ -4856,20 +4856,10 @@
       <c r="D60" s="11">
         <v>-1</v>
       </c>
-      <c r="E60" s="29"/>
+      <c r="E60" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="E58:E60"/>
-    <mergeCell ref="E52:E55"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E14:E16"/>
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="E19:E22"/>
     <mergeCell ref="E40:E43"/>
@@ -4878,6 +4868,16 @@
     <mergeCell ref="E23:E27"/>
     <mergeCell ref="E28:E31"/>
     <mergeCell ref="E32:E35"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="E52:E55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
delivery slot addition updated
</commit_message>
<xml_diff>
--- a/src/main/resources/ClientPortal_Data.xlsx
+++ b/src/main/resources/ClientPortal_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BS01361\My Folder\0. Test Type\4. Automation Testing\Selenium Files\MAS_FloraFire\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1BFD2C-D3FA-4774-B731-DCC354703090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{291D10F7-3355-40E6-9355-6081FDDC3A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="803" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" tabRatio="803" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Value" sheetId="2" r:id="rId1"/>
@@ -21,8 +21,8 @@
     <sheet name="GiftCard" sheetId="10" r:id="rId6"/>
     <sheet name="Employee" sheetId="12" r:id="rId7"/>
     <sheet name="Zone" sheetId="13" r:id="rId8"/>
-    <sheet name="Slot" sheetId="15" r:id="rId9"/>
-    <sheet name="Mode" sheetId="17" r:id="rId10"/>
+    <sheet name="Mode" sheetId="17" r:id="rId9"/>
+    <sheet name="Slot" sheetId="15" r:id="rId10"/>
     <sheet name="Calendar" sheetId="21" r:id="rId11"/>
     <sheet name="Code" sheetId="16" r:id="rId12"/>
     <sheet name="ShortCode" sheetId="19" r:id="rId13"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1201" uniqueCount="575">
   <si>
     <t>Name</t>
   </si>
@@ -1239,9 +1239,6 @@
     <t>Slot1</t>
   </si>
   <si>
-    <t>Slot2</t>
-  </si>
-  <si>
     <t>Mode Name</t>
   </si>
   <si>
@@ -1759,6 +1756,15 @@
   </si>
   <si>
     <t>Renault Trafic</t>
+  </si>
+  <si>
+    <t>Garland Road</t>
+  </si>
+  <si>
+    <t>DS-EVE</t>
+  </si>
+  <si>
+    <t>02</t>
   </si>
 </sst>
 </file>
@@ -2132,19 +2138,19 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2589,7 +2595,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B20" s="2">
         <v>18</v>
@@ -2597,7 +2603,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B21" s="2">
         <v>19</v>
@@ -2610,50 +2616,81 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5DA318D-8073-4D46-A062-C668992104C1}">
-  <dimension ref="A1:C3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA816B9A-A2BD-448E-99B5-2B148B525D17}">
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="14" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="8.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" style="17" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" style="17" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>400</v>
+        <v>383</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>385</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>386</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>391</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>392</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>397</v>
-      </c>
       <c r="B3" s="2" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>390</v>
+        <v>90</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>394</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>392</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>395</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
@@ -2671,15 +2708,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>505</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>506</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>396</v>
@@ -2722,310 +2759,310 @@
   <sheetData>
     <row r="1" spans="1:14" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>202</v>
       </c>
       <c r="C1" s="13" t="s">
+        <v>401</v>
+      </c>
+      <c r="D1" s="13" t="s">
         <v>402</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>403</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>404</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>405</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="H1" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="I1" s="13" t="s">
         <v>406</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>407</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>408</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>409</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>410</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>411</v>
-      </c>
-      <c r="N1" s="13" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>419</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>420</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L2" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>421</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>91</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>91</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>91</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>
@@ -3067,7 +3104,7 @@
         <v>144</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>85</v>
@@ -3091,27 +3128,27 @@
         <v>97</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="K1" s="13" t="s">
+        <v>477</v>
+      </c>
+      <c r="L1" s="13" t="s">
         <v>478</v>
-      </c>
-      <c r="L1" s="13" t="s">
-        <v>479</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>21</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>99</v>
@@ -3132,10 +3169,10 @@
         <v>90001</v>
       </c>
       <c r="I2" s="15" t="s">
+        <v>490</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>491</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>492</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>45</v>
@@ -3152,10 +3189,10 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>114</v>
@@ -3176,10 +3213,10 @@
         <v>78701</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>45</v>
@@ -3196,10 +3233,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>121</v>
@@ -3218,10 +3255,10 @@
         <v>75201</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>45</v>
@@ -3238,10 +3275,10 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>128</v>
@@ -3262,10 +3299,10 @@
         <v>10118</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>45</v>
@@ -3282,10 +3319,10 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>135</v>
@@ -3306,10 +3343,10 @@
         <v>60606</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>45</v>
@@ -3381,7 +3418,7 @@
         <v>171</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>177</v>
@@ -3404,7 +3441,7 @@
         <v>172</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>178</v>
@@ -3427,7 +3464,7 @@
         <v>173</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>179</v>
@@ -3450,7 +3487,7 @@
         <v>174</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>180</v>
@@ -3473,7 +3510,7 @@
         <v>175</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>181</v>
@@ -3496,7 +3533,7 @@
         <v>176</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>182</v>
@@ -3786,12 +3823,12 @@
         <v>268</v>
       </c>
       <c r="AM1" s="13" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="2" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>60</v>
@@ -3800,19 +3837,19 @@
         <v>29</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>58</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="G2" s="23" t="s">
         <v>55</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>262</v>
@@ -3827,7 +3864,7 @@
         <v>90</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="N2" s="15" t="s">
         <v>253</v>
@@ -3892,7 +3929,7 @@
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="23" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AM2" s="23" t="s">
         <v>91</v>
@@ -3947,7 +3984,7 @@
       <c r="D2" s="8">
         <v>1</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="27" t="s">
         <v>81</v>
       </c>
     </row>
@@ -3964,7 +4001,7 @@
       <c r="D3" s="2">
         <v>0</v>
       </c>
-      <c r="E3" s="29"/>
+      <c r="E3" s="28"/>
     </row>
     <row r="4" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
@@ -3979,7 +4016,7 @@
       <c r="D4" s="11">
         <v>-1</v>
       </c>
-      <c r="E4" s="26"/>
+      <c r="E4" s="29"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -3994,7 +4031,7 @@
       <c r="D5" s="8">
         <v>1</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="27" t="s">
         <v>82</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -4014,7 +4051,7 @@
       <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6" s="29"/>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
@@ -4029,7 +4066,7 @@
       <c r="D7" s="6">
         <v>-1</v>
       </c>
-      <c r="E7" s="26"/>
+      <c r="E7" s="29"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -4044,7 +4081,7 @@
       <c r="D8" s="8">
         <v>1</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="27" t="s">
         <v>83</v>
       </c>
     </row>
@@ -4061,7 +4098,7 @@
       <c r="D9" s="2">
         <v>0</v>
       </c>
-      <c r="E9" s="29"/>
+      <c r="E9" s="28"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
@@ -4076,7 +4113,7 @@
       <c r="D10" s="2">
         <v>0</v>
       </c>
-      <c r="E10" s="29"/>
+      <c r="E10" s="28"/>
     </row>
     <row r="11" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
@@ -4091,7 +4128,7 @@
       <c r="D11" s="6">
         <v>-1</v>
       </c>
-      <c r="E11" s="29"/>
+      <c r="E11" s="28"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -4106,7 +4143,7 @@
       <c r="D12" s="8">
         <v>1</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="27" t="s">
         <v>68</v>
       </c>
     </row>
@@ -4123,7 +4160,7 @@
       <c r="D13" s="11">
         <v>-1</v>
       </c>
-      <c r="E13" s="26"/>
+      <c r="E13" s="29"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
@@ -4138,7 +4175,7 @@
       <c r="D14" s="8">
         <v>1</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="27" t="s">
         <v>69</v>
       </c>
     </row>
@@ -4155,7 +4192,7 @@
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="E15" s="29"/>
+      <c r="E15" s="28"/>
     </row>
     <row r="16" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
@@ -4170,7 +4207,7 @@
       <c r="D16" s="6">
         <v>-1</v>
       </c>
-      <c r="E16" s="26"/>
+      <c r="E16" s="29"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
@@ -4185,7 +4222,7 @@
       <c r="D17" s="8">
         <v>1</v>
       </c>
-      <c r="E17" s="25" t="s">
+      <c r="E17" s="27" t="s">
         <v>70</v>
       </c>
     </row>
@@ -4202,7 +4239,7 @@
       <c r="D18" s="11">
         <v>-1</v>
       </c>
-      <c r="E18" s="26"/>
+      <c r="E18" s="29"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
@@ -4217,7 +4254,7 @@
       <c r="D19" s="8">
         <v>1</v>
       </c>
-      <c r="E19" s="25" t="s">
+      <c r="E19" s="27" t="s">
         <v>71</v>
       </c>
     </row>
@@ -4234,7 +4271,7 @@
       <c r="D20" s="2">
         <v>0</v>
       </c>
-      <c r="E20" s="29"/>
+      <c r="E20" s="28"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
@@ -4249,7 +4286,7 @@
       <c r="D21" s="2">
         <v>0</v>
       </c>
-      <c r="E21" s="29"/>
+      <c r="E21" s="28"/>
     </row>
     <row r="22" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
@@ -4264,7 +4301,7 @@
       <c r="D22" s="6">
         <v>-1</v>
       </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="29"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
@@ -4279,7 +4316,7 @@
       <c r="D23" s="8">
         <v>1</v>
       </c>
-      <c r="E23" s="25" t="s">
+      <c r="E23" s="27" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4296,7 +4333,7 @@
       <c r="D24" s="2">
         <v>0</v>
       </c>
-      <c r="E24" s="29"/>
+      <c r="E24" s="28"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
@@ -4311,7 +4348,7 @@
       <c r="D25" s="2">
         <v>0</v>
       </c>
-      <c r="E25" s="29"/>
+      <c r="E25" s="28"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
@@ -4326,7 +4363,7 @@
       <c r="D26" s="2">
         <v>0</v>
       </c>
-      <c r="E26" s="29"/>
+      <c r="E26" s="28"/>
     </row>
     <row r="27" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
@@ -4341,7 +4378,7 @@
       <c r="D27" s="11">
         <v>-1</v>
       </c>
-      <c r="E27" s="26"/>
+      <c r="E27" s="29"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
@@ -4356,7 +4393,7 @@
       <c r="D28" s="8">
         <v>1</v>
       </c>
-      <c r="E28" s="25" t="s">
+      <c r="E28" s="27" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4373,7 +4410,7 @@
       <c r="D29" s="2">
         <v>0</v>
       </c>
-      <c r="E29" s="29"/>
+      <c r="E29" s="28"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
@@ -4388,7 +4425,7 @@
       <c r="D30" s="2">
         <v>0</v>
       </c>
-      <c r="E30" s="29"/>
+      <c r="E30" s="28"/>
     </row>
     <row r="31" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
@@ -4403,7 +4440,7 @@
       <c r="D31" s="6">
         <v>-1</v>
       </c>
-      <c r="E31" s="26"/>
+      <c r="E31" s="29"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
@@ -4418,7 +4455,7 @@
       <c r="D32" s="8">
         <v>1</v>
       </c>
-      <c r="E32" s="25" t="s">
+      <c r="E32" s="27" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4435,7 +4472,7 @@
       <c r="D33" s="2">
         <v>0</v>
       </c>
-      <c r="E33" s="29"/>
+      <c r="E33" s="28"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
@@ -4450,7 +4487,7 @@
       <c r="D34" s="2">
         <v>0</v>
       </c>
-      <c r="E34" s="29"/>
+      <c r="E34" s="28"/>
     </row>
     <row r="35" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
@@ -4465,7 +4502,7 @@
       <c r="D35" s="6">
         <v>-1</v>
       </c>
-      <c r="E35" s="26"/>
+      <c r="E35" s="29"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
@@ -4480,7 +4517,7 @@
       <c r="D36" s="8">
         <v>1</v>
       </c>
-      <c r="E36" s="25" t="s">
+      <c r="E36" s="27" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4497,7 +4534,7 @@
       <c r="D37" s="11">
         <v>-1</v>
       </c>
-      <c r="E37" s="26"/>
+      <c r="E37" s="29"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
@@ -4512,7 +4549,7 @@
       <c r="D38" s="8">
         <v>1</v>
       </c>
-      <c r="E38" s="25" t="s">
+      <c r="E38" s="27" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4529,7 +4566,7 @@
       <c r="D39" s="11">
         <v>-1</v>
       </c>
-      <c r="E39" s="26"/>
+      <c r="E39" s="29"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
@@ -4544,7 +4581,7 @@
       <c r="D40" s="8">
         <v>1</v>
       </c>
-      <c r="E40" s="25" t="s">
+      <c r="E40" s="27" t="s">
         <v>77</v>
       </c>
     </row>
@@ -4561,7 +4598,7 @@
       <c r="D41" s="2">
         <v>0</v>
       </c>
-      <c r="E41" s="29"/>
+      <c r="E41" s="28"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
@@ -4576,7 +4613,7 @@
       <c r="D42" s="2">
         <v>0</v>
       </c>
-      <c r="E42" s="29"/>
+      <c r="E42" s="28"/>
     </row>
     <row r="43" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
@@ -4591,7 +4628,7 @@
       <c r="D43" s="6">
         <v>-1</v>
       </c>
-      <c r="E43" s="26"/>
+      <c r="E43" s="29"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
@@ -4606,7 +4643,7 @@
       <c r="D44" s="8">
         <v>1</v>
       </c>
-      <c r="E44" s="25" t="s">
+      <c r="E44" s="27" t="s">
         <v>78</v>
       </c>
     </row>
@@ -4623,7 +4660,7 @@
       <c r="D45" s="2">
         <v>0</v>
       </c>
-      <c r="E45" s="29"/>
+      <c r="E45" s="28"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
@@ -4638,7 +4675,7 @@
       <c r="D46" s="2">
         <v>0</v>
       </c>
-      <c r="E46" s="29"/>
+      <c r="E46" s="28"/>
     </row>
     <row r="47" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
@@ -4653,7 +4690,7 @@
       <c r="D47" s="6">
         <v>-1</v>
       </c>
-      <c r="E47" s="26"/>
+      <c r="E47" s="29"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
@@ -4668,7 +4705,7 @@
       <c r="D48" s="8">
         <v>1</v>
       </c>
-      <c r="E48" s="25" t="s">
+      <c r="E48" s="27" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4685,7 +4722,7 @@
       <c r="D49" s="2">
         <v>0</v>
       </c>
-      <c r="E49" s="29"/>
+      <c r="E49" s="28"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
@@ -4700,7 +4737,7 @@
       <c r="D50" s="2">
         <v>0</v>
       </c>
-      <c r="E50" s="29"/>
+      <c r="E50" s="28"/>
     </row>
     <row r="51" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
@@ -4715,7 +4752,7 @@
       <c r="D51" s="6">
         <v>-1</v>
       </c>
-      <c r="E51" s="26"/>
+      <c r="E51" s="29"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
@@ -4730,7 +4767,7 @@
       <c r="D52" s="8">
         <v>1</v>
       </c>
-      <c r="E52" s="25" t="s">
+      <c r="E52" s="27" t="s">
         <v>80</v>
       </c>
     </row>
@@ -4747,7 +4784,7 @@
       <c r="D53" s="2">
         <v>0</v>
       </c>
-      <c r="E53" s="29"/>
+      <c r="E53" s="28"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
@@ -4762,7 +4799,7 @@
       <c r="D54" s="2">
         <v>0</v>
       </c>
-      <c r="E54" s="29"/>
+      <c r="E54" s="28"/>
     </row>
     <row r="55" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="12" t="s">
@@ -4777,11 +4814,11 @@
       <c r="D55" s="6">
         <v>-1</v>
       </c>
-      <c r="E55" s="29"/>
+      <c r="E55" s="28"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B56" s="8">
         <v>0</v>
@@ -4792,13 +4829,13 @@
       <c r="D56" s="8">
         <v>1</v>
       </c>
-      <c r="E56" s="27" t="s">
-        <v>498</v>
+      <c r="E56" s="25" t="s">
+        <v>497</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="12" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B57" s="6">
         <v>1</v>
@@ -4809,11 +4846,11 @@
       <c r="D57" s="6">
         <v>-1</v>
       </c>
-      <c r="E57" s="28"/>
+      <c r="E57" s="26"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B58" s="8">
         <v>0</v>
@@ -4824,13 +4861,13 @@
       <c r="D58" s="8">
         <v>1</v>
       </c>
-      <c r="E58" s="25" t="s">
-        <v>499</v>
+      <c r="E58" s="27" t="s">
+        <v>498</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B59" s="2">
         <v>1</v>
@@ -4841,11 +4878,11 @@
       <c r="D59" s="2">
         <v>0</v>
       </c>
-      <c r="E59" s="29"/>
+      <c r="E59" s="28"/>
     </row>
     <row r="60" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B60" s="11">
         <v>2</v>
@@ -4856,10 +4893,20 @@
       <c r="D60" s="11">
         <v>-1</v>
       </c>
-      <c r="E60" s="26"/>
+      <c r="E60" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="E52:E55"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E14:E16"/>
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="E19:E22"/>
     <mergeCell ref="E40:E43"/>
@@ -4868,16 +4915,6 @@
     <mergeCell ref="E23:E27"/>
     <mergeCell ref="E28:E31"/>
     <mergeCell ref="E32:E35"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="E58:E60"/>
-    <mergeCell ref="E52:E55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
@@ -5006,7 +5043,7 @@
         <v>25</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>91</v>
@@ -5066,7 +5103,7 @@
         <v>25</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>3</v>
@@ -5087,7 +5124,7 @@
         <v>104</v>
       </c>
       <c r="S3" s="14" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="T3" s="15" t="s">
         <v>112</v>
@@ -5126,7 +5163,7 @@
         <v>140</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>91</v>
@@ -5182,7 +5219,7 @@
         <v>25</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>3</v>
@@ -5242,7 +5279,7 @@
         <v>140</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>91</v>
@@ -5302,7 +5339,7 @@
         <v>25</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>3</v>
@@ -5508,7 +5545,7 @@
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>61</v>
@@ -5517,19 +5554,19 @@
         <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="G2" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>262</v>
@@ -5544,7 +5581,7 @@
         <v>1</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="N2" s="15" t="s">
         <v>253</v>
@@ -5609,12 +5646,12 @@
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>61</v>
@@ -5623,19 +5660,19 @@
         <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>55</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="I3" s="15" t="s">
         <v>262</v>
@@ -5650,7 +5687,7 @@
         <v>1</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="N3" s="15" t="s">
         <v>253</v>
@@ -5715,7 +5752,7 @@
       </c>
       <c r="AK3" s="23"/>
       <c r="AL3" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.3">
@@ -5732,7 +5769,7 @@
         <v>239</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="F4" s="24" t="s">
         <v>243</v>
@@ -5817,10 +5854,10 @@
         <v>91</v>
       </c>
       <c r="AH4" s="22" t="s">
+        <v>549</v>
+      </c>
+      <c r="AI4" s="22" t="s">
         <v>550</v>
-      </c>
-      <c r="AI4" s="22" t="s">
-        <v>551</v>
       </c>
       <c r="AJ4" s="15" t="s">
         <v>3</v>
@@ -5844,7 +5881,7 @@
         <v>240</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>244</v>
@@ -5927,10 +5964,10 @@
         <v>91</v>
       </c>
       <c r="AH5" s="22" t="s">
+        <v>549</v>
+      </c>
+      <c r="AI5" s="22" t="s">
         <v>550</v>
-      </c>
-      <c r="AI5" s="22" t="s">
-        <v>551</v>
       </c>
       <c r="AJ5" s="15" t="s">
         <v>3</v>
@@ -5951,7 +5988,7 @@
         <v>29</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>57</v>
@@ -6037,10 +6074,10 @@
         <v>91</v>
       </c>
       <c r="AH6" s="22" t="s">
+        <v>549</v>
+      </c>
+      <c r="AI6" s="22" t="s">
         <v>550</v>
-      </c>
-      <c r="AI6" s="22" t="s">
-        <v>551</v>
       </c>
       <c r="AJ6" s="15" t="s">
         <v>3</v>
@@ -6061,7 +6098,7 @@
         <v>29</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>57</v>
@@ -6149,10 +6186,10 @@
         <v>91</v>
       </c>
       <c r="AH7" s="22" t="s">
+        <v>549</v>
+      </c>
+      <c r="AI7" s="22" t="s">
         <v>550</v>
-      </c>
-      <c r="AI7" s="22" t="s">
-        <v>551</v>
       </c>
       <c r="AJ7" s="15" t="s">
         <v>3</v>
@@ -6167,7 +6204,7 @@
         <v>238</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>29</v>
@@ -6176,7 +6213,7 @@
         <v>241</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F8" s="19" t="s">
         <v>247</v>
@@ -6270,7 +6307,7 @@
     </row>
     <row r="9" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>372</v>
@@ -6279,19 +6316,19 @@
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>372</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>262</v>
@@ -6306,7 +6343,7 @@
         <v>1</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="N9" s="15" t="s">
         <v>253</v>
@@ -6371,12 +6408,12 @@
       </c>
       <c r="AK9" s="2"/>
       <c r="AL9" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>372</v>
@@ -6385,19 +6422,19 @@
         <v>29</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>372</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>261</v>
@@ -6412,7 +6449,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="N10" s="15" t="s">
         <v>253</v>
@@ -6477,51 +6514,51 @@
       </c>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H11" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>557</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>558</v>
       </c>
       <c r="J11" s="2">
         <v>1</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="L11" s="2">
         <v>1</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="O11" s="19" t="s">
         <v>3</v>
@@ -6583,33 +6620,33 @@
       </c>
       <c r="AK11" s="15"/>
       <c r="AL11" s="15" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="12" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>261</v>
@@ -6624,10 +6661,10 @@
         <v>1</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="O12" s="19" t="s">
         <v>3</v>
@@ -6689,7 +6726,7 @@
       </c>
       <c r="AK12" s="15"/>
       <c r="AL12" s="15" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
   </sheetData>
@@ -6973,7 +7010,7 @@
         <v>1001</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D2" s="20" t="s">
         <v>283</v>
@@ -7017,7 +7054,7 @@
         <v>1003</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>283</v>
@@ -7766,81 +7803,86 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA816B9A-A2BD-448E-99B5-2B148B525D17}">
-  <dimension ref="A1:F3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5DA318D-8073-4D46-A062-C668992104C1}">
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="14" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" style="17" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" style="17" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="14.5546875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>383</v>
+        <v>399</v>
       </c>
       <c r="B1" s="13" t="s">
+        <v>398</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>384</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>385</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>386</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>387</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>378</v>
-      </c>
       <c r="C2" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="E2" s="15" t="s">
         <v>391</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="F2" s="15" t="s">
         <v>392</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="G2" s="15" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>378</v>
+        <v>573</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="15" t="s">
-        <v>394</v>
-      </c>
       <c r="E3" s="15" t="s">
+        <v>574</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>392</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="G3" s="15" t="s">
         <v>395</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
customer page element updated
</commit_message>
<xml_diff>
--- a/src/main/resources/ClientPortal_Data.xlsx
+++ b/src/main/resources/ClientPortal_Data.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BS01361\My Folder\0. Test Type\4. Automation Testing\Selenium Files\MAS_FloraFire\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{889CF8C8-8031-49E3-8617-30CDB2E854F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA447AE2-0C91-40BD-B4FC-B39CC282F316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="803" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" tabRatio="803" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Value" sheetId="2" r:id="rId1"/>
     <sheet name="ValueList" sheetId="1" r:id="rId2"/>
-    <sheet name="Customer" sheetId="4" r:id="rId3"/>
+    <sheet name="Customer" sheetId="23" r:id="rId3"/>
     <sheet name="Product" sheetId="8" r:id="rId4"/>
     <sheet name="Discount" sheetId="11" r:id="rId5"/>
     <sheet name="GiftCard" sheetId="10" r:id="rId6"/>
@@ -2159,19 +2159,19 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4005,7 +4005,7 @@
       <c r="D2" s="8">
         <v>1</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="26" t="s">
         <v>81</v>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
       <c r="D3" s="2">
         <v>0</v>
       </c>
-      <c r="E3" s="29"/>
+      <c r="E3" s="28"/>
     </row>
     <row r="4" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
@@ -4037,7 +4037,7 @@
       <c r="D4" s="11">
         <v>-1</v>
       </c>
-      <c r="E4" s="30"/>
+      <c r="E4" s="27"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -4052,7 +4052,7 @@
       <c r="D5" s="8">
         <v>1</v>
       </c>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="26" t="s">
         <v>82</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -4072,7 +4072,7 @@
       <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6" s="29"/>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
@@ -4087,7 +4087,7 @@
       <c r="D7" s="6">
         <v>-1</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="27"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -4102,7 +4102,7 @@
       <c r="D8" s="8">
         <v>1</v>
       </c>
-      <c r="E8" s="28" t="s">
+      <c r="E8" s="26" t="s">
         <v>83</v>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
       <c r="D9" s="2">
         <v>0</v>
       </c>
-      <c r="E9" s="29"/>
+      <c r="E9" s="28"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
@@ -4134,7 +4134,7 @@
       <c r="D10" s="2">
         <v>0</v>
       </c>
-      <c r="E10" s="29"/>
+      <c r="E10" s="28"/>
     </row>
     <row r="11" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
@@ -4149,7 +4149,7 @@
       <c r="D11" s="6">
         <v>-1</v>
       </c>
-      <c r="E11" s="29"/>
+      <c r="E11" s="28"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -4164,7 +4164,7 @@
       <c r="D12" s="8">
         <v>1</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="26" t="s">
         <v>68</v>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       <c r="D13" s="11">
         <v>-1</v>
       </c>
-      <c r="E13" s="30"/>
+      <c r="E13" s="27"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
@@ -4196,7 +4196,7 @@
       <c r="D14" s="8">
         <v>1</v>
       </c>
-      <c r="E14" s="28" t="s">
+      <c r="E14" s="26" t="s">
         <v>69</v>
       </c>
     </row>
@@ -4213,7 +4213,7 @@
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="E15" s="29"/>
+      <c r="E15" s="28"/>
     </row>
     <row r="16" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
@@ -4228,7 +4228,7 @@
       <c r="D16" s="6">
         <v>-1</v>
       </c>
-      <c r="E16" s="30"/>
+      <c r="E16" s="27"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
@@ -4243,7 +4243,7 @@
       <c r="D17" s="8">
         <v>1</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E17" s="26" t="s">
         <v>70</v>
       </c>
     </row>
@@ -4260,7 +4260,7 @@
       <c r="D18" s="11">
         <v>-1</v>
       </c>
-      <c r="E18" s="30"/>
+      <c r="E18" s="27"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
@@ -4275,7 +4275,7 @@
       <c r="D19" s="8">
         <v>1</v>
       </c>
-      <c r="E19" s="28" t="s">
+      <c r="E19" s="26" t="s">
         <v>71</v>
       </c>
     </row>
@@ -4292,7 +4292,7 @@
       <c r="D20" s="2">
         <v>0</v>
       </c>
-      <c r="E20" s="29"/>
+      <c r="E20" s="28"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
@@ -4307,7 +4307,7 @@
       <c r="D21" s="2">
         <v>0</v>
       </c>
-      <c r="E21" s="29"/>
+      <c r="E21" s="28"/>
     </row>
     <row r="22" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
@@ -4322,7 +4322,7 @@
       <c r="D22" s="6">
         <v>-1</v>
       </c>
-      <c r="E22" s="30"/>
+      <c r="E22" s="27"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
@@ -4337,7 +4337,7 @@
       <c r="D23" s="8">
         <v>1</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E23" s="26" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4354,7 +4354,7 @@
       <c r="D24" s="2">
         <v>0</v>
       </c>
-      <c r="E24" s="29"/>
+      <c r="E24" s="28"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
@@ -4369,7 +4369,7 @@
       <c r="D25" s="2">
         <v>0</v>
       </c>
-      <c r="E25" s="29"/>
+      <c r="E25" s="28"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
@@ -4384,7 +4384,7 @@
       <c r="D26" s="2">
         <v>0</v>
       </c>
-      <c r="E26" s="29"/>
+      <c r="E26" s="28"/>
     </row>
     <row r="27" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
@@ -4399,7 +4399,7 @@
       <c r="D27" s="11">
         <v>-1</v>
       </c>
-      <c r="E27" s="30"/>
+      <c r="E27" s="27"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
@@ -4414,7 +4414,7 @@
       <c r="D28" s="8">
         <v>1</v>
       </c>
-      <c r="E28" s="28" t="s">
+      <c r="E28" s="26" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       <c r="D29" s="2">
         <v>0</v>
       </c>
-      <c r="E29" s="29"/>
+      <c r="E29" s="28"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
@@ -4446,7 +4446,7 @@
       <c r="D30" s="2">
         <v>0</v>
       </c>
-      <c r="E30" s="29"/>
+      <c r="E30" s="28"/>
     </row>
     <row r="31" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
@@ -4461,7 +4461,7 @@
       <c r="D31" s="6">
         <v>-1</v>
       </c>
-      <c r="E31" s="30"/>
+      <c r="E31" s="27"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
@@ -4476,7 +4476,7 @@
       <c r="D32" s="8">
         <v>1</v>
       </c>
-      <c r="E32" s="28" t="s">
+      <c r="E32" s="26" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4493,7 +4493,7 @@
       <c r="D33" s="2">
         <v>0</v>
       </c>
-      <c r="E33" s="29"/>
+      <c r="E33" s="28"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
@@ -4508,7 +4508,7 @@
       <c r="D34" s="2">
         <v>0</v>
       </c>
-      <c r="E34" s="29"/>
+      <c r="E34" s="28"/>
     </row>
     <row r="35" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
@@ -4523,7 +4523,7 @@
       <c r="D35" s="6">
         <v>-1</v>
       </c>
-      <c r="E35" s="30"/>
+      <c r="E35" s="27"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
@@ -4538,7 +4538,7 @@
       <c r="D36" s="8">
         <v>1</v>
       </c>
-      <c r="E36" s="28" t="s">
+      <c r="E36" s="26" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       <c r="D37" s="11">
         <v>-1</v>
       </c>
-      <c r="E37" s="30"/>
+      <c r="E37" s="27"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
@@ -4570,7 +4570,7 @@
       <c r="D38" s="8">
         <v>1</v>
       </c>
-      <c r="E38" s="28" t="s">
+      <c r="E38" s="26" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       <c r="D39" s="11">
         <v>-1</v>
       </c>
-      <c r="E39" s="30"/>
+      <c r="E39" s="27"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
@@ -4602,7 +4602,7 @@
       <c r="D40" s="8">
         <v>1</v>
       </c>
-      <c r="E40" s="28" t="s">
+      <c r="E40" s="26" t="s">
         <v>77</v>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       <c r="D41" s="2">
         <v>0</v>
       </c>
-      <c r="E41" s="29"/>
+      <c r="E41" s="28"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
@@ -4634,7 +4634,7 @@
       <c r="D42" s="2">
         <v>0</v>
       </c>
-      <c r="E42" s="29"/>
+      <c r="E42" s="28"/>
     </row>
     <row r="43" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
@@ -4649,7 +4649,7 @@
       <c r="D43" s="6">
         <v>-1</v>
       </c>
-      <c r="E43" s="30"/>
+      <c r="E43" s="27"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
@@ -4664,7 +4664,7 @@
       <c r="D44" s="8">
         <v>1</v>
       </c>
-      <c r="E44" s="28" t="s">
+      <c r="E44" s="26" t="s">
         <v>78</v>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       <c r="D45" s="2">
         <v>0</v>
       </c>
-      <c r="E45" s="29"/>
+      <c r="E45" s="28"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
@@ -4696,7 +4696,7 @@
       <c r="D46" s="2">
         <v>0</v>
       </c>
-      <c r="E46" s="29"/>
+      <c r="E46" s="28"/>
     </row>
     <row r="47" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
@@ -4711,7 +4711,7 @@
       <c r="D47" s="6">
         <v>-1</v>
       </c>
-      <c r="E47" s="30"/>
+      <c r="E47" s="27"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
@@ -4726,7 +4726,7 @@
       <c r="D48" s="8">
         <v>1</v>
       </c>
-      <c r="E48" s="28" t="s">
+      <c r="E48" s="26" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4743,7 +4743,7 @@
       <c r="D49" s="2">
         <v>0</v>
       </c>
-      <c r="E49" s="29"/>
+      <c r="E49" s="28"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
@@ -4758,7 +4758,7 @@
       <c r="D50" s="2">
         <v>0</v>
       </c>
-      <c r="E50" s="29"/>
+      <c r="E50" s="28"/>
     </row>
     <row r="51" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
@@ -4773,7 +4773,7 @@
       <c r="D51" s="6">
         <v>-1</v>
       </c>
-      <c r="E51" s="30"/>
+      <c r="E51" s="27"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
@@ -4788,7 +4788,7 @@
       <c r="D52" s="8">
         <v>1</v>
       </c>
-      <c r="E52" s="28" t="s">
+      <c r="E52" s="26" t="s">
         <v>80</v>
       </c>
     </row>
@@ -4805,7 +4805,7 @@
       <c r="D53" s="2">
         <v>0</v>
       </c>
-      <c r="E53" s="29"/>
+      <c r="E53" s="28"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
@@ -4820,7 +4820,7 @@
       <c r="D54" s="2">
         <v>0</v>
       </c>
-      <c r="E54" s="29"/>
+      <c r="E54" s="28"/>
     </row>
     <row r="55" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="12" t="s">
@@ -4835,7 +4835,7 @@
       <c r="D55" s="6">
         <v>-1</v>
       </c>
-      <c r="E55" s="29"/>
+      <c r="E55" s="28"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
@@ -4850,7 +4850,7 @@
       <c r="D56" s="8">
         <v>1</v>
       </c>
-      <c r="E56" s="26" t="s">
+      <c r="E56" s="29" t="s">
         <v>492</v>
       </c>
     </row>
@@ -4867,7 +4867,7 @@
       <c r="D57" s="6">
         <v>-1</v>
       </c>
-      <c r="E57" s="27"/>
+      <c r="E57" s="30"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
@@ -4882,7 +4882,7 @@
       <c r="D58" s="8">
         <v>1</v>
       </c>
-      <c r="E58" s="28" t="s">
+      <c r="E58" s="26" t="s">
         <v>493</v>
       </c>
     </row>
@@ -4899,7 +4899,7 @@
       <c r="D59" s="2">
         <v>0</v>
       </c>
-      <c r="E59" s="29"/>
+      <c r="E59" s="28"/>
     </row>
     <row r="60" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
@@ -4914,12 +4914,10 @@
       <c r="D60" s="11">
         <v>-1</v>
       </c>
-      <c r="E60" s="30"/>
+      <c r="E60" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="E38:E39"/>
     <mergeCell ref="E56:E57"/>
     <mergeCell ref="E58:E60"/>
     <mergeCell ref="E52:E55"/>
@@ -4936,6 +4934,8 @@
     <mergeCell ref="E23:E27"/>
     <mergeCell ref="E28:E31"/>
     <mergeCell ref="E32:E35"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="E38:E39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
@@ -4943,7 +4943,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75B8A7D-056B-43CF-B8CF-47A9850E51E0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2B7E47-44AB-4DB1-9135-930A58432CC4}">
   <dimension ref="A1:T7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5389,12 +5389,12 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="S3" r:id="rId1" xr:uid="{FAFBBC17-1F1F-4CE2-BBF2-E4AEA8EE1ED4}"/>
-    <hyperlink ref="S4" r:id="rId2" xr:uid="{F3C188DE-CC3C-4EF9-8248-BB75D6CA48C5}"/>
-    <hyperlink ref="S5" r:id="rId3" xr:uid="{3162BC19-B05A-40BA-92BD-54B8E669E299}"/>
-    <hyperlink ref="S6" r:id="rId4" xr:uid="{93615EC5-2AF1-4B5B-9A79-A890026A7F9E}"/>
-    <hyperlink ref="S7" r:id="rId5" xr:uid="{904212DF-3581-4833-B3AE-9EB777FD795F}"/>
-    <hyperlink ref="S2" r:id="rId6" xr:uid="{429C311D-6D48-48CA-9A9D-C04FAC21AFC1}"/>
+    <hyperlink ref="S3" r:id="rId1" xr:uid="{2F49A58A-274E-4DED-83D7-843E6442001B}"/>
+    <hyperlink ref="S4" r:id="rId2" xr:uid="{776ACF63-7866-45CA-A13C-2E83F97458CE}"/>
+    <hyperlink ref="S5" r:id="rId3" xr:uid="{89EF0D0E-5A2C-4CA2-BCA1-35691BAB869C}"/>
+    <hyperlink ref="S6" r:id="rId4" xr:uid="{A3AC07BE-AFD5-4142-924C-77926AB827E3}"/>
+    <hyperlink ref="S7" r:id="rId5" xr:uid="{2851FD21-D7BA-42D4-BD48-593503DDAEA4}"/>
+    <hyperlink ref="S2" r:id="rId6" xr:uid="{CFD3E0EA-9797-4BD0-9367-AE64A0D5ABAE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId7"/>

</xml_diff>

<commit_message>
product page element updated
</commit_message>
<xml_diff>
--- a/src/main/resources/ClientPortal_Data.xlsx
+++ b/src/main/resources/ClientPortal_Data.xlsx
@@ -8,27 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BS01361\My Folder\0. Test Type\4. Automation Testing\Selenium Files\MAS_FloraFire\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA447AE2-0C91-40BD-B4FC-B39CC282F316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F24F05-2681-499C-8287-CA4CC5B7B3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" tabRatio="803" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" tabRatio="803" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Value" sheetId="2" r:id="rId1"/>
     <sheet name="ValueList" sheetId="1" r:id="rId2"/>
     <sheet name="Customer" sheetId="23" r:id="rId3"/>
-    <sheet name="Product" sheetId="8" r:id="rId4"/>
-    <sheet name="Discount" sheetId="11" r:id="rId5"/>
-    <sheet name="GiftCard" sheetId="10" r:id="rId6"/>
-    <sheet name="Employee" sheetId="12" r:id="rId7"/>
-    <sheet name="Zone" sheetId="13" r:id="rId8"/>
-    <sheet name="Mode" sheetId="17" r:id="rId9"/>
-    <sheet name="Slot" sheetId="15" r:id="rId10"/>
-    <sheet name="Calendar" sheetId="21" r:id="rId11"/>
-    <sheet name="Code" sheetId="16" r:id="rId12"/>
-    <sheet name="ShortCode" sheetId="19" r:id="rId13"/>
-    <sheet name="Vehicle" sheetId="7" r:id="rId14"/>
-    <sheet name="ShortCuts" sheetId="6" r:id="rId15"/>
-    <sheet name="Test" sheetId="22" r:id="rId16"/>
+    <sheet name="Product" sheetId="24" r:id="rId4"/>
+    <sheet name="Product (2)" sheetId="25" r:id="rId5"/>
+    <sheet name="Discount" sheetId="11" r:id="rId6"/>
+    <sheet name="GiftCard" sheetId="10" r:id="rId7"/>
+    <sheet name="Employee" sheetId="12" r:id="rId8"/>
+    <sheet name="Zone" sheetId="13" r:id="rId9"/>
+    <sheet name="Mode" sheetId="17" r:id="rId10"/>
+    <sheet name="Slot" sheetId="15" r:id="rId11"/>
+    <sheet name="Calendar" sheetId="21" r:id="rId12"/>
+    <sheet name="Code" sheetId="16" r:id="rId13"/>
+    <sheet name="ShortCode" sheetId="19" r:id="rId14"/>
+    <sheet name="Vehicle" sheetId="7" r:id="rId15"/>
+    <sheet name="ShortCuts" sheetId="6" r:id="rId16"/>
+    <sheet name="Test" sheetId="22" r:id="rId17"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1311" uniqueCount="582">
   <si>
     <t>Name</t>
   </si>
@@ -891,9 +892,6 @@
     <t>5/31/2025</t>
   </si>
   <si>
-    <t>6/30/2025</t>
-  </si>
-  <si>
     <t>Amount</t>
   </si>
   <si>
@@ -1783,6 +1781,12 @@
   </si>
   <si>
     <t>manager</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>5</t>
   </si>
 </sst>
 </file>
@@ -2165,13 +2169,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2616,7 +2620,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B20" s="2">
         <v>18</v>
@@ -2624,7 +2628,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B21" s="2">
         <v>19</v>
@@ -2637,6 +2641,92 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5DA318D-8073-4D46-A062-C668992104C1}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>392</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>378</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>379</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>380</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>385</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>568</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>389</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA816B9A-A2BD-448E-99B5-2B148B525D17}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -2652,62 +2742,62 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>378</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>380</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>381</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>382</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D2" s="15" t="s">
+        <v>385</v>
+      </c>
+      <c r="E2" s="15" t="s">
         <v>386</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="F2" s="15" t="s">
         <v>387</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D3" s="15" t="s">
+        <v>388</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>389</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>387</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>390</v>
       </c>
     </row>
   </sheetData>
@@ -2717,7 +2807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F571E0E-8389-463F-9299-88D0F2C4674B}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -2729,18 +2819,18 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>498</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>499</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -2748,7 +2838,7 @@
         <v>264</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -2757,7 +2847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08473418-9C08-4415-9A18-E4B9858BD3EF}">
   <dimension ref="A1:N7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -2780,310 +2870,310 @@
   <sheetData>
     <row r="1" spans="1:14" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>202</v>
       </c>
       <c r="C1" s="13" t="s">
+        <v>395</v>
+      </c>
+      <c r="D1" s="13" t="s">
         <v>396</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>397</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>398</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>399</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="H1" s="13" t="s">
+        <v>399</v>
+      </c>
+      <c r="I1" s="13" t="s">
         <v>400</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>401</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>402</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>403</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>405</v>
-      </c>
-      <c r="N1" s="13" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>413</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>414</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L2" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>415</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>91</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>91</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>91</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
   </sheetData>
@@ -3098,7 +3188,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0917F802-0E2D-4130-BB01-3BF4DABE74A1}">
   <dimension ref="A1:N6"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -3125,7 +3215,7 @@
         <v>144</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>85</v>
@@ -3149,27 +3239,27 @@
         <v>97</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="K1" s="13" t="s">
+        <v>471</v>
+      </c>
+      <c r="L1" s="13" t="s">
         <v>472</v>
-      </c>
-      <c r="L1" s="13" t="s">
-        <v>473</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>21</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>99</v>
@@ -3190,16 +3280,16 @@
         <v>90001</v>
       </c>
       <c r="I2" s="15" t="s">
+        <v>484</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>485</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>486</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>3</v>
@@ -3210,10 +3300,10 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>114</v>
@@ -3234,10 +3324,10 @@
         <v>78701</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>45</v>
@@ -3254,10 +3344,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>121</v>
@@ -3276,16 +3366,16 @@
         <v>75201</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>3</v>
@@ -3296,10 +3386,10 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>128</v>
@@ -3320,10 +3410,10 @@
         <v>10118</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>45</v>
@@ -3340,10 +3430,10 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>135</v>
@@ -3364,16 +3454,16 @@
         <v>60606</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>91</v>
@@ -3396,7 +3486,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE96B074-BAA6-41E4-A885-01589CFEB352}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -3439,7 +3529,7 @@
         <v>171</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>177</v>
@@ -3462,7 +3552,7 @@
         <v>172</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>178</v>
@@ -3485,7 +3575,7 @@
         <v>173</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>179</v>
@@ -3508,7 +3598,7 @@
         <v>174</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>180</v>
@@ -3531,7 +3621,7 @@
         <v>175</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>181</v>
@@ -3554,7 +3644,7 @@
         <v>176</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>182</v>
@@ -3578,7 +3668,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F28B997F-3DC4-4C7D-9993-70026FD21600}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -3682,7 +3772,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{570EFCBF-8E1B-4B5B-AD83-ED4683CA7299}">
   <dimension ref="A1:AM2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -3844,12 +3934,12 @@
         <v>268</v>
       </c>
       <c r="AM1" s="13" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="2" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>60</v>
@@ -3858,19 +3948,19 @@
         <v>29</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>58</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="G2" s="23" t="s">
         <v>55</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>262</v>
@@ -3885,7 +3975,7 @@
         <v>90</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="N2" s="15" t="s">
         <v>253</v>
@@ -3950,7 +4040,7 @@
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="23" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="AM2" s="23" t="s">
         <v>91</v>
@@ -4022,7 +4112,7 @@
       <c r="D3" s="2">
         <v>0</v>
       </c>
-      <c r="E3" s="28"/>
+      <c r="E3" s="30"/>
     </row>
     <row r="4" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
@@ -4072,7 +4162,7 @@
       <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6" s="28"/>
+      <c r="E6" s="30"/>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
@@ -4119,7 +4209,7 @@
       <c r="D9" s="2">
         <v>0</v>
       </c>
-      <c r="E9" s="28"/>
+      <c r="E9" s="30"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
@@ -4134,7 +4224,7 @@
       <c r="D10" s="2">
         <v>0</v>
       </c>
-      <c r="E10" s="28"/>
+      <c r="E10" s="30"/>
     </row>
     <row r="11" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
@@ -4149,7 +4239,7 @@
       <c r="D11" s="6">
         <v>-1</v>
       </c>
-      <c r="E11" s="28"/>
+      <c r="E11" s="30"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -4213,7 +4303,7 @@
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="E15" s="28"/>
+      <c r="E15" s="30"/>
     </row>
     <row r="16" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
@@ -4292,7 +4382,7 @@
       <c r="D20" s="2">
         <v>0</v>
       </c>
-      <c r="E20" s="28"/>
+      <c r="E20" s="30"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
@@ -4307,7 +4397,7 @@
       <c r="D21" s="2">
         <v>0</v>
       </c>
-      <c r="E21" s="28"/>
+      <c r="E21" s="30"/>
     </row>
     <row r="22" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
@@ -4354,7 +4444,7 @@
       <c r="D24" s="2">
         <v>0</v>
       </c>
-      <c r="E24" s="28"/>
+      <c r="E24" s="30"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
@@ -4369,7 +4459,7 @@
       <c r="D25" s="2">
         <v>0</v>
       </c>
-      <c r="E25" s="28"/>
+      <c r="E25" s="30"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
@@ -4384,7 +4474,7 @@
       <c r="D26" s="2">
         <v>0</v>
       </c>
-      <c r="E26" s="28"/>
+      <c r="E26" s="30"/>
     </row>
     <row r="27" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
@@ -4431,7 +4521,7 @@
       <c r="D29" s="2">
         <v>0</v>
       </c>
-      <c r="E29" s="28"/>
+      <c r="E29" s="30"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
@@ -4446,7 +4536,7 @@
       <c r="D30" s="2">
         <v>0</v>
       </c>
-      <c r="E30" s="28"/>
+      <c r="E30" s="30"/>
     </row>
     <row r="31" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
@@ -4493,11 +4583,11 @@
       <c r="D33" s="2">
         <v>0</v>
       </c>
-      <c r="E33" s="28"/>
+      <c r="E33" s="30"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B34" s="2">
         <v>2</v>
@@ -4508,7 +4598,7 @@
       <c r="D34" s="2">
         <v>0</v>
       </c>
-      <c r="E34" s="28"/>
+      <c r="E34" s="30"/>
     </row>
     <row r="35" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
@@ -4619,7 +4709,7 @@
       <c r="D41" s="2">
         <v>0</v>
       </c>
-      <c r="E41" s="28"/>
+      <c r="E41" s="30"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
@@ -4634,7 +4724,7 @@
       <c r="D42" s="2">
         <v>0</v>
       </c>
-      <c r="E42" s="28"/>
+      <c r="E42" s="30"/>
     </row>
     <row r="43" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
@@ -4681,7 +4771,7 @@
       <c r="D45" s="2">
         <v>0</v>
       </c>
-      <c r="E45" s="28"/>
+      <c r="E45" s="30"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
@@ -4696,7 +4786,7 @@
       <c r="D46" s="2">
         <v>0</v>
       </c>
-      <c r="E46" s="28"/>
+      <c r="E46" s="30"/>
     </row>
     <row r="47" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
@@ -4743,7 +4833,7 @@
       <c r="D49" s="2">
         <v>0</v>
       </c>
-      <c r="E49" s="28"/>
+      <c r="E49" s="30"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
@@ -4758,7 +4848,7 @@
       <c r="D50" s="2">
         <v>0</v>
       </c>
-      <c r="E50" s="28"/>
+      <c r="E50" s="30"/>
     </row>
     <row r="51" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
@@ -4805,7 +4895,7 @@
       <c r="D53" s="2">
         <v>0</v>
       </c>
-      <c r="E53" s="28"/>
+      <c r="E53" s="30"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
@@ -4820,7 +4910,7 @@
       <c r="D54" s="2">
         <v>0</v>
       </c>
-      <c r="E54" s="28"/>
+      <c r="E54" s="30"/>
     </row>
     <row r="55" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="12" t="s">
@@ -4835,11 +4925,11 @@
       <c r="D55" s="6">
         <v>-1</v>
       </c>
-      <c r="E55" s="28"/>
+      <c r="E55" s="30"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B56" s="8">
         <v>0</v>
@@ -4850,13 +4940,13 @@
       <c r="D56" s="8">
         <v>1</v>
       </c>
-      <c r="E56" s="29" t="s">
-        <v>492</v>
+      <c r="E56" s="28" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="12" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B57" s="6">
         <v>1</v>
@@ -4867,11 +4957,11 @@
       <c r="D57" s="6">
         <v>-1</v>
       </c>
-      <c r="E57" s="30"/>
+      <c r="E57" s="29"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B58" s="8">
         <v>0</v>
@@ -4883,12 +4973,12 @@
         <v>1</v>
       </c>
       <c r="E58" s="26" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B59" s="2">
         <v>1</v>
@@ -4899,11 +4989,11 @@
       <c r="D59" s="2">
         <v>0</v>
       </c>
-      <c r="E59" s="28"/>
+      <c r="E59" s="30"/>
     </row>
     <row r="60" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B60" s="11">
         <v>2</v>
@@ -4918,14 +5008,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="E58:E60"/>
-    <mergeCell ref="E52:E55"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E14:E16"/>
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="E19:E22"/>
     <mergeCell ref="E40:E43"/>
@@ -4934,8 +5016,16 @@
     <mergeCell ref="E23:E27"/>
     <mergeCell ref="E28:E31"/>
     <mergeCell ref="E32:E35"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E14:E16"/>
     <mergeCell ref="E36:E37"/>
     <mergeCell ref="E38:E39"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="E52:E55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
@@ -5064,7 +5154,7 @@
         <v>25</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>91</v>
@@ -5124,7 +5214,7 @@
         <v>25</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>3</v>
@@ -5145,7 +5235,7 @@
         <v>104</v>
       </c>
       <c r="S3" s="14" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="T3" s="15" t="s">
         <v>112</v>
@@ -5184,7 +5274,7 @@
         <v>140</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>91</v>
@@ -5240,7 +5330,7 @@
         <v>25</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>3</v>
@@ -5300,7 +5390,7 @@
         <v>140</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>91</v>
@@ -5360,7 +5450,7 @@
         <v>25</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>3</v>
@@ -5402,7 +5492,388 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C76421E-550A-4F58-ABC5-0AC68C5F2DE6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE083F72-6C0E-4564-830C-AF36FA19A4AA}">
+  <dimension ref="A1:AL3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" style="17" customWidth="1"/>
+    <col min="6" max="6" width="27.33203125" style="17" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="77.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.33203125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.109375" style="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="14.6640625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="21.6640625" style="1" customWidth="1"/>
+    <col min="34" max="34" width="12.109375" style="1" customWidth="1"/>
+    <col min="35" max="35" width="12" style="1" customWidth="1"/>
+    <col min="36" max="36" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="5.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="13.5546875" style="1" customWidth="1"/>
+    <col min="39" max="39" width="8.88671875" style="1" customWidth="1"/>
+    <col min="40" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:38" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="L1" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="M1" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="N1" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="O1" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="S1" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="T1" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="U1" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="V1" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="W1" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="X1" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="Y1" s="13" t="s">
+        <v>221</v>
+      </c>
+      <c r="Z1" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="AA1" s="13" t="s">
+        <v>223</v>
+      </c>
+      <c r="AB1" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="AC1" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="AD1" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="AE1" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="AF1" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="AG1" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="AH1" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="AI1" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="AJ1" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="AK1" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="AL1" s="13" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>549</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>546</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="L2" s="2">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="O2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="P2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="S2" s="2">
+        <v>14.99</v>
+      </c>
+      <c r="T2" s="2">
+        <v>17.989999999999998</v>
+      </c>
+      <c r="U2" s="2">
+        <v>19.989999999999998</v>
+      </c>
+      <c r="V2" s="2">
+        <v>12.99</v>
+      </c>
+      <c r="W2" s="2">
+        <v>30</v>
+      </c>
+      <c r="X2" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y2" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z2" s="2">
+        <v>50</v>
+      </c>
+      <c r="AA2" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="15" t="s">
+        <v>580</v>
+      </c>
+      <c r="AC2" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF2" s="20"/>
+      <c r="AG2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH2" s="21"/>
+      <c r="AI2" s="21"/>
+      <c r="AJ2" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="AK2" s="15"/>
+      <c r="AL2" s="15" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>556</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>553</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>261</v>
+      </c>
+      <c r="J3" s="2">
+        <v>1</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>261</v>
+      </c>
+      <c r="L3" s="2">
+        <v>1</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="O3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="P3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="S3" s="2">
+        <v>12.99</v>
+      </c>
+      <c r="T3" s="2">
+        <v>15.99</v>
+      </c>
+      <c r="U3" s="2">
+        <v>19.989999999999998</v>
+      </c>
+      <c r="V3" s="2">
+        <v>13.99</v>
+      </c>
+      <c r="W3" s="2">
+        <v>50</v>
+      </c>
+      <c r="X3" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y3" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z3" s="2">
+        <v>15</v>
+      </c>
+      <c r="AA3" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="15" t="s">
+        <v>581</v>
+      </c>
+      <c r="AC3" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF3" s="20"/>
+      <c r="AG3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH3" s="21"/>
+      <c r="AI3" s="21"/>
+      <c r="AJ3" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="AK3" s="15"/>
+      <c r="AL3" s="15" t="s">
+        <v>559</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{303FC3B1-B557-4227-BB56-3144CCBBF032}">
   <dimension ref="A1:AL12"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5566,7 +6037,7 @@
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>61</v>
@@ -5575,19 +6046,19 @@
         <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="G2" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>262</v>
@@ -5602,7 +6073,7 @@
         <v>1</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="N2" s="15" t="s">
         <v>253</v>
@@ -5645,7 +6116,7 @@
         <v>0</v>
       </c>
       <c r="AB2" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AC2" s="19" t="s">
         <v>3</v>
@@ -5667,12 +6138,12 @@
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>61</v>
@@ -5681,19 +6152,19 @@
         <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>55</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="I3" s="15" t="s">
         <v>262</v>
@@ -5708,7 +6179,7 @@
         <v>1</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="N3" s="15" t="s">
         <v>253</v>
@@ -5751,7 +6222,7 @@
         <v>0</v>
       </c>
       <c r="AB3" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AC3" s="19" t="s">
         <v>3</v>
@@ -5773,7 +6244,7 @@
       </c>
       <c r="AK3" s="23"/>
       <c r="AL3" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.3">
@@ -5790,7 +6261,7 @@
         <v>239</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="F4" s="24" t="s">
         <v>243</v>
@@ -5857,7 +6328,7 @@
         <v>263</v>
       </c>
       <c r="AB4" s="15" t="s">
-        <v>263</v>
+        <v>580</v>
       </c>
       <c r="AC4" s="15" t="s">
         <v>91</v>
@@ -5875,10 +6346,10 @@
         <v>91</v>
       </c>
       <c r="AH4" s="22" t="s">
+        <v>543</v>
+      </c>
+      <c r="AI4" s="22" t="s">
         <v>544</v>
-      </c>
-      <c r="AI4" s="22" t="s">
-        <v>545</v>
       </c>
       <c r="AJ4" s="15" t="s">
         <v>3</v>
@@ -5902,7 +6373,7 @@
         <v>240</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>244</v>
@@ -5969,7 +6440,7 @@
         <v>263</v>
       </c>
       <c r="AB5" s="15" t="s">
-        <v>263</v>
+        <v>580</v>
       </c>
       <c r="AC5" s="15" t="s">
         <v>91</v>
@@ -5985,10 +6456,10 @@
         <v>91</v>
       </c>
       <c r="AH5" s="22" t="s">
+        <v>543</v>
+      </c>
+      <c r="AI5" s="22" t="s">
         <v>544</v>
-      </c>
-      <c r="AI5" s="22" t="s">
-        <v>545</v>
       </c>
       <c r="AJ5" s="15" t="s">
         <v>3</v>
@@ -6009,7 +6480,7 @@
         <v>29</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>57</v>
@@ -6079,7 +6550,7 @@
         <v>263</v>
       </c>
       <c r="AB6" s="15" t="s">
-        <v>263</v>
+        <v>580</v>
       </c>
       <c r="AC6" s="15" t="s">
         <v>91</v>
@@ -6095,10 +6566,10 @@
         <v>91</v>
       </c>
       <c r="AH6" s="22" t="s">
+        <v>543</v>
+      </c>
+      <c r="AI6" s="22" t="s">
         <v>544</v>
-      </c>
-      <c r="AI6" s="22" t="s">
-        <v>545</v>
       </c>
       <c r="AJ6" s="15" t="s">
         <v>3</v>
@@ -6119,7 +6590,7 @@
         <v>29</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>57</v>
@@ -6189,7 +6660,7 @@
         <v>263</v>
       </c>
       <c r="AB7" s="15" t="s">
-        <v>263</v>
+        <v>580</v>
       </c>
       <c r="AC7" s="15" t="s">
         <v>91</v>
@@ -6207,10 +6678,10 @@
         <v>91</v>
       </c>
       <c r="AH7" s="22" t="s">
+        <v>543</v>
+      </c>
+      <c r="AI7" s="22" t="s">
         <v>544</v>
-      </c>
-      <c r="AI7" s="22" t="s">
-        <v>545</v>
       </c>
       <c r="AJ7" s="15" t="s">
         <v>3</v>
@@ -6225,7 +6696,7 @@
         <v>238</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>29</v>
@@ -6234,7 +6705,7 @@
         <v>241</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F8" s="19" t="s">
         <v>247</v>
@@ -6301,7 +6772,7 @@
         <v>263</v>
       </c>
       <c r="AB8" s="15" t="s">
-        <v>263</v>
+        <v>580</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>91</v>
@@ -6328,28 +6799,28 @@
     </row>
     <row r="9" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>262</v>
@@ -6364,7 +6835,7 @@
         <v>1</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="N9" s="15" t="s">
         <v>253</v>
@@ -6407,7 +6878,7 @@
         <v>263</v>
       </c>
       <c r="AB9" s="15" t="s">
-        <v>263</v>
+        <v>580</v>
       </c>
       <c r="AC9" s="19" t="s">
         <v>3</v>
@@ -6429,33 +6900,33 @@
       </c>
       <c r="AK9" s="2"/>
       <c r="AL9" s="2" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>261</v>
@@ -6470,7 +6941,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="N10" s="15" t="s">
         <v>253</v>
@@ -6513,7 +6984,7 @@
         <v>263</v>
       </c>
       <c r="AB10" s="15" t="s">
-        <v>263</v>
+        <v>580</v>
       </c>
       <c r="AC10" s="19" t="s">
         <v>3</v>
@@ -6535,51 +7006,51 @@
       </c>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H11" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>551</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>552</v>
       </c>
       <c r="J11" s="2">
         <v>1</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L11" s="2">
         <v>1</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="O11" s="19" t="s">
         <v>3</v>
@@ -6618,8 +7089,8 @@
       <c r="AA11" s="2">
         <v>0</v>
       </c>
-      <c r="AB11" s="2">
-        <v>0</v>
+      <c r="AB11" s="15" t="s">
+        <v>580</v>
       </c>
       <c r="AC11" s="15" t="s">
         <v>91</v>
@@ -6641,33 +7112,33 @@
       </c>
       <c r="AK11" s="15"/>
       <c r="AL11" s="15" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="12" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>261</v>
@@ -6682,10 +7153,10 @@
         <v>1</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="O12" s="19" t="s">
         <v>3</v>
@@ -6724,8 +7195,8 @@
       <c r="AA12" s="2">
         <v>0</v>
       </c>
-      <c r="AB12" s="2">
-        <v>0</v>
+      <c r="AB12" s="15" t="s">
+        <v>581</v>
       </c>
       <c r="AC12" s="15" t="s">
         <v>91</v>
@@ -6747,17 +7218,16 @@
       </c>
       <c r="AK12" s="15"/>
       <c r="AL12" s="15" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F147CD6B-CA39-477C-82FD-5D86870A8EFB}">
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -6780,7 +7250,7 @@
         <v>126</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D1" s="13" t="s">
         <v>141</v>
@@ -6789,7 +7259,7 @@
         <v>231</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>209</v>
@@ -6797,10 +7267,10 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C2" s="19">
         <v>30</v>
@@ -6812,18 +7282,18 @@
         <v>282</v>
       </c>
       <c r="F2" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C3" s="1">
         <v>10</v>
@@ -6832,44 +7302,44 @@
         <v>29</v>
       </c>
       <c r="E3" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>296</v>
-      </c>
-      <c r="F3" s="19" t="s">
-        <v>291</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
+        <v>287</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>288</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>289</v>
       </c>
       <c r="C4" s="19">
         <v>20</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E4" s="20" t="s">
         <v>282</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C5" s="19">
         <v>5</v>
@@ -6884,15 +7354,15 @@
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C6" s="19">
         <v>50</v>
@@ -6907,15 +7377,15 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C7" s="19">
         <v>10</v>
@@ -6930,15 +7400,15 @@
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C8" s="19">
         <v>100</v>
@@ -6950,18 +7420,18 @@
         <v>282</v>
       </c>
       <c r="F8" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>303</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C9" s="19">
         <v>100</v>
@@ -6973,10 +7443,10 @@
         <v>282</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -6986,7 +7456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C6C325F-4A76-431C-998A-38D75363C07E}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -7031,10 +7501,10 @@
         <v>1001</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>283</v>
+        <v>544</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>29</v>
@@ -7055,7 +7525,7 @@
         <v>53</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>282</v>
+        <v>544</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>62</v>
@@ -7075,10 +7545,10 @@
         <v>1003</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>283</v>
+        <v>544</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>32</v>
@@ -7096,7 +7566,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C7655F-AC18-4255-9C9F-28DEDD520460}">
   <dimension ref="A1:W9"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -7127,10 +7597,10 @@
   <sheetData>
     <row r="1" spans="1:23" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>306</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>307</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>308</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>85</v>
@@ -7151,7 +7621,7 @@
         <v>90</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J1" s="13" t="s">
         <v>97</v>
@@ -7160,48 +7630,48 @@
         <v>96</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="O1" s="13" t="s">
         <v>202</v>
       </c>
       <c r="P1" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="Q1" s="13" t="s">
         <v>312</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>313</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>314</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>317</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="W1" s="13" t="s">
         <v>318</v>
-      </c>
-      <c r="W1" s="13" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
+        <v>319</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>320</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>321</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>99</v>
@@ -7222,16 +7692,16 @@
         <v>90001</v>
       </c>
       <c r="I2" s="15" t="s">
+        <v>321</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="K2" s="15" t="s">
         <v>322</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="L2" s="15" t="s">
         <v>324</v>
-      </c>
-      <c r="K2" s="15" t="s">
-        <v>323</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>325</v>
       </c>
       <c r="M2" s="19" t="s">
         <v>29</v>
@@ -7246,33 +7716,33 @@
         <v>91</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="R2" s="15" t="s">
+        <v>325</v>
+      </c>
+      <c r="S2" s="15" t="s">
         <v>326</v>
       </c>
-      <c r="S2" s="15" t="s">
+      <c r="T2" s="15" t="s">
         <v>327</v>
-      </c>
-      <c r="T2" s="15" t="s">
-        <v>328</v>
       </c>
       <c r="U2" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="W2" s="19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
+        <v>329</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>330</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>331</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>114</v>
@@ -7293,16 +7763,16 @@
         <v>78701</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="M3" s="19" t="s">
         <v>29</v>
@@ -7317,33 +7787,33 @@
         <v>91</v>
       </c>
       <c r="Q3" s="19" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="R3" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="S3" s="15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="T3" s="15" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="U3" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V3" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="W3" s="19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>121</v>
@@ -7362,16 +7832,16 @@
         <v>75201</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="M4" s="19" t="s">
         <v>62</v>
@@ -7386,33 +7856,33 @@
         <v>91</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="R4" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="S4" s="15" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="T4" s="15" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="U4" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="W4" s="19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
+        <v>344</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>345</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>346</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>128</v>
@@ -7433,22 +7903,22 @@
         <v>10118</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="M5" s="19" t="s">
         <v>29</v>
       </c>
       <c r="N5" s="19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="O5" s="15" t="s">
         <v>47</v>
@@ -7457,33 +7927,33 @@
         <v>91</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="R5" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="S5" s="15" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="T5" s="15" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="U5" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="W5" s="19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
+        <v>346</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>347</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>348</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>135</v>
@@ -7504,16 +7974,16 @@
         <v>60606</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="M6" s="19" t="s">
         <v>29</v>
@@ -7528,33 +7998,33 @@
         <v>3</v>
       </c>
       <c r="Q6" s="19" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="R6" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="S6" s="15" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="T6" s="15" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="U6" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="W6" s="19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
+        <v>569</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>570</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>571</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>135</v>
@@ -7575,22 +8045,22 @@
         <v>60606</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="M7" s="19" t="s">
         <v>29</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="O7" s="15" t="s">
         <v>47</v>
@@ -7599,25 +8069,25 @@
         <v>3</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="R7" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="S7" s="15" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="T7" s="15" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="U7" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V7" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="W7" s="19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.3">
@@ -7657,7 +8127,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3846B3E9-78EC-4A21-B7B1-295C9A6CBED2}">
   <dimension ref="A1:V5"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -7685,7 +8155,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>209</v>
@@ -7694,81 +8164,81 @@
         <v>126</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>353</v>
+      </c>
+      <c r="E1" s="13" t="s">
         <v>354</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>355</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>356</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="H1" s="13" t="s">
         <v>357</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="I1" s="13" t="s">
         <v>358</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>359</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>360</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>361</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>362</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>363</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="O1" s="13" t="s">
         <v>364</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="P1" s="13" t="s">
         <v>365</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="Q1" s="13" t="s">
         <v>366</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>367</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>368</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>369</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>370</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>371</v>
-      </c>
-      <c r="V1" s="13" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>373</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>374</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>140</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E2" s="15" t="s">
+        <v>375</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>376</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>377</v>
       </c>
       <c r="G2" s="2">
         <v>23.7044</v>
@@ -7822,13 +8292,13 @@
         <v>90</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>140</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="15"/>
@@ -7890,90 +8360,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5DA318D-8073-4D46-A062-C668992104C1}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
-        <v>394</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>393</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>379</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>380</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>382</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>567</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>386</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>387</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>568</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>567</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>569</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>387</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>390</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
corporate settings page element updated
</commit_message>
<xml_diff>
--- a/src/main/resources/ClientPortal_Data.xlsx
+++ b/src/main/resources/ClientPortal_Data.xlsx
@@ -8,28 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BS01361\My Folder\0. Test Type\4. Automation Testing\Selenium Files\MAS_FloraFire\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F24F05-2681-499C-8287-CA4CC5B7B3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBC2282-2245-4C8C-8A15-61B6626FDC8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" tabRatio="803" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" tabRatio="803" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Value" sheetId="2" r:id="rId1"/>
     <sheet name="ValueList" sheetId="1" r:id="rId2"/>
     <sheet name="Customer" sheetId="23" r:id="rId3"/>
-    <sheet name="Product" sheetId="24" r:id="rId4"/>
-    <sheet name="Product (2)" sheetId="25" r:id="rId5"/>
-    <sheet name="Discount" sheetId="11" r:id="rId6"/>
-    <sheet name="GiftCard" sheetId="10" r:id="rId7"/>
-    <sheet name="Employee" sheetId="12" r:id="rId8"/>
-    <sheet name="Zone" sheetId="13" r:id="rId9"/>
-    <sheet name="Mode" sheetId="17" r:id="rId10"/>
-    <sheet name="Slot" sheetId="15" r:id="rId11"/>
-    <sheet name="Calendar" sheetId="21" r:id="rId12"/>
-    <sheet name="Code" sheetId="16" r:id="rId13"/>
-    <sheet name="ShortCode" sheetId="19" r:id="rId14"/>
-    <sheet name="Vehicle" sheetId="7" r:id="rId15"/>
-    <sheet name="ShortCuts" sheetId="6" r:id="rId16"/>
-    <sheet name="Test" sheetId="22" r:id="rId17"/>
+    <sheet name="Product" sheetId="25" r:id="rId4"/>
+    <sheet name="Discount" sheetId="11" r:id="rId5"/>
+    <sheet name="GiftCard" sheetId="10" r:id="rId6"/>
+    <sheet name="Employee" sheetId="12" r:id="rId7"/>
+    <sheet name="Zone" sheetId="13" r:id="rId8"/>
+    <sheet name="Mode" sheetId="17" r:id="rId9"/>
+    <sheet name="Slot" sheetId="15" r:id="rId10"/>
+    <sheet name="Calendar" sheetId="21" r:id="rId11"/>
+    <sheet name="Code" sheetId="16" r:id="rId12"/>
+    <sheet name="ShortCode" sheetId="19" r:id="rId13"/>
+    <sheet name="Vehicle" sheetId="7" r:id="rId14"/>
+    <sheet name="ShortCuts" sheetId="6" r:id="rId15"/>
+    <sheet name="Test" sheetId="22" r:id="rId16"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1311" uniqueCount="582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1225" uniqueCount="580">
   <si>
     <t>Name</t>
   </si>
@@ -889,9 +888,6 @@
     <t>Promotional</t>
   </si>
   <si>
-    <t>5/31/2025</t>
-  </si>
-  <si>
     <t>Amount</t>
   </si>
   <si>
@@ -926,9 +922,6 @@
   </si>
   <si>
     <t>FLOWER10</t>
-  </si>
-  <si>
-    <t>5/31/2026</t>
   </si>
   <si>
     <t>10% off on all flower bouquets.</t>
@@ -2163,19 +2156,19 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2620,7 +2613,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B20" s="2">
         <v>18</v>
@@ -2628,7 +2621,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="B21" s="2">
         <v>19</v>
@@ -2641,92 +2634,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5DA318D-8073-4D46-A062-C668992104C1}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
-        <v>393</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>392</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>378</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>379</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>380</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>385</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>386</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>567</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>568</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>386</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>389</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA816B9A-A2BD-448E-99B5-2B148B525D17}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -2742,62 +2649,62 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>376</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>377</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>378</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>380</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D2" s="15" t="s">
+        <v>383</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>385</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>386</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -2807,7 +2714,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F571E0E-8389-463F-9299-88D0F2C4674B}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -2819,18 +2726,18 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -2838,7 +2745,7 @@
         <v>264</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>
@@ -2847,7 +2754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08473418-9C08-4415-9A18-E4B9858BD3EF}">
   <dimension ref="A1:N7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -2870,310 +2777,310 @@
   <sheetData>
     <row r="1" spans="1:14" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>202</v>
       </c>
       <c r="C1" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>394</v>
+      </c>
+      <c r="E1" s="13" t="s">
         <v>395</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>396</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>397</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>398</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="H1" s="13" t="s">
+        <v>397</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>398</v>
+      </c>
+      <c r="J1" s="13" t="s">
         <v>399</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>400</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>401</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>402</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>403</v>
-      </c>
-      <c r="M1" s="13" t="s">
-        <v>404</v>
-      </c>
-      <c r="N1" s="13" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>411</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>413</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>440</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>442</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>91</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>446</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>448</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>91</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>91</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
   </sheetData>
@@ -3188,7 +3095,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0917F802-0E2D-4130-BB01-3BF4DABE74A1}">
   <dimension ref="A1:N6"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -3215,7 +3122,7 @@
         <v>144</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>85</v>
@@ -3239,27 +3146,27 @@
         <v>97</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>21</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>99</v>
@@ -3280,16 +3187,16 @@
         <v>90001</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>3</v>
@@ -3300,10 +3207,10 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>114</v>
@@ -3324,10 +3231,10 @@
         <v>78701</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>45</v>
@@ -3344,10 +3251,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>121</v>
@@ -3366,16 +3273,16 @@
         <v>75201</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>3</v>
@@ -3386,10 +3293,10 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>128</v>
@@ -3410,10 +3317,10 @@
         <v>10118</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>45</v>
@@ -3430,10 +3337,10 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>135</v>
@@ -3454,16 +3361,16 @@
         <v>60606</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>91</v>
@@ -3486,7 +3393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE96B074-BAA6-41E4-A885-01589CFEB352}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -3529,7 +3436,7 @@
         <v>171</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>177</v>
@@ -3552,7 +3459,7 @@
         <v>172</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>178</v>
@@ -3575,7 +3482,7 @@
         <v>173</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>179</v>
@@ -3598,7 +3505,7 @@
         <v>174</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>180</v>
@@ -3621,7 +3528,7 @@
         <v>175</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>181</v>
@@ -3644,7 +3551,7 @@
         <v>176</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>182</v>
@@ -3668,7 +3575,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F28B997F-3DC4-4C7D-9993-70026FD21600}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -3772,7 +3679,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{570EFCBF-8E1B-4B5B-AD83-ED4683CA7299}">
   <dimension ref="A1:AM2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -3934,12 +3841,12 @@
         <v>268</v>
       </c>
       <c r="AM1" s="13" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
     </row>
     <row r="2" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>60</v>
@@ -3948,19 +3855,19 @@
         <v>29</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>58</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="G2" s="23" t="s">
         <v>55</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>262</v>
@@ -3975,7 +3882,7 @@
         <v>90</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="N2" s="15" t="s">
         <v>253</v>
@@ -4040,7 +3947,7 @@
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="23" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="AM2" s="23" t="s">
         <v>91</v>
@@ -4095,7 +4002,7 @@
       <c r="D2" s="8">
         <v>1</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="28" t="s">
         <v>81</v>
       </c>
     </row>
@@ -4112,7 +4019,7 @@
       <c r="D3" s="2">
         <v>0</v>
       </c>
-      <c r="E3" s="30"/>
+      <c r="E3" s="29"/>
     </row>
     <row r="4" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
@@ -4127,7 +4034,7 @@
       <c r="D4" s="11">
         <v>-1</v>
       </c>
-      <c r="E4" s="27"/>
+      <c r="E4" s="30"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -4142,7 +4049,7 @@
       <c r="D5" s="8">
         <v>1</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="E5" s="28" t="s">
         <v>82</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -4162,7 +4069,7 @@
       <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
@@ -4177,7 +4084,7 @@
       <c r="D7" s="6">
         <v>-1</v>
       </c>
-      <c r="E7" s="27"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -4192,7 +4099,7 @@
       <c r="D8" s="8">
         <v>1</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="28" t="s">
         <v>83</v>
       </c>
     </row>
@@ -4209,7 +4116,7 @@
       <c r="D9" s="2">
         <v>0</v>
       </c>
-      <c r="E9" s="30"/>
+      <c r="E9" s="29"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
@@ -4224,7 +4131,7 @@
       <c r="D10" s="2">
         <v>0</v>
       </c>
-      <c r="E10" s="30"/>
+      <c r="E10" s="29"/>
     </row>
     <row r="11" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
@@ -4239,7 +4146,7 @@
       <c r="D11" s="6">
         <v>-1</v>
       </c>
-      <c r="E11" s="30"/>
+      <c r="E11" s="29"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -4254,7 +4161,7 @@
       <c r="D12" s="8">
         <v>1</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="28" t="s">
         <v>68</v>
       </c>
     </row>
@@ -4271,7 +4178,7 @@
       <c r="D13" s="11">
         <v>-1</v>
       </c>
-      <c r="E13" s="27"/>
+      <c r="E13" s="30"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
@@ -4286,7 +4193,7 @@
       <c r="D14" s="8">
         <v>1</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="28" t="s">
         <v>69</v>
       </c>
     </row>
@@ -4303,7 +4210,7 @@
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="E15" s="30"/>
+      <c r="E15" s="29"/>
     </row>
     <row r="16" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
@@ -4318,7 +4225,7 @@
       <c r="D16" s="6">
         <v>-1</v>
       </c>
-      <c r="E16" s="27"/>
+      <c r="E16" s="30"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
@@ -4333,7 +4240,7 @@
       <c r="D17" s="8">
         <v>1</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="28" t="s">
         <v>70</v>
       </c>
     </row>
@@ -4350,7 +4257,7 @@
       <c r="D18" s="11">
         <v>-1</v>
       </c>
-      <c r="E18" s="27"/>
+      <c r="E18" s="30"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
@@ -4365,7 +4272,7 @@
       <c r="D19" s="8">
         <v>1</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="28" t="s">
         <v>71</v>
       </c>
     </row>
@@ -4382,7 +4289,7 @@
       <c r="D20" s="2">
         <v>0</v>
       </c>
-      <c r="E20" s="30"/>
+      <c r="E20" s="29"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
@@ -4397,7 +4304,7 @@
       <c r="D21" s="2">
         <v>0</v>
       </c>
-      <c r="E21" s="30"/>
+      <c r="E21" s="29"/>
     </row>
     <row r="22" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
@@ -4412,7 +4319,7 @@
       <c r="D22" s="6">
         <v>-1</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="30"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
@@ -4427,7 +4334,7 @@
       <c r="D23" s="8">
         <v>1</v>
       </c>
-      <c r="E23" s="26" t="s">
+      <c r="E23" s="28" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4444,7 +4351,7 @@
       <c r="D24" s="2">
         <v>0</v>
       </c>
-      <c r="E24" s="30"/>
+      <c r="E24" s="29"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
@@ -4459,7 +4366,7 @@
       <c r="D25" s="2">
         <v>0</v>
       </c>
-      <c r="E25" s="30"/>
+      <c r="E25" s="29"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
@@ -4474,7 +4381,7 @@
       <c r="D26" s="2">
         <v>0</v>
       </c>
-      <c r="E26" s="30"/>
+      <c r="E26" s="29"/>
     </row>
     <row r="27" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
@@ -4489,7 +4396,7 @@
       <c r="D27" s="11">
         <v>-1</v>
       </c>
-      <c r="E27" s="27"/>
+      <c r="E27" s="30"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
@@ -4504,7 +4411,7 @@
       <c r="D28" s="8">
         <v>1</v>
       </c>
-      <c r="E28" s="26" t="s">
+      <c r="E28" s="28" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4521,7 +4428,7 @@
       <c r="D29" s="2">
         <v>0</v>
       </c>
-      <c r="E29" s="30"/>
+      <c r="E29" s="29"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
@@ -4536,7 +4443,7 @@
       <c r="D30" s="2">
         <v>0</v>
       </c>
-      <c r="E30" s="30"/>
+      <c r="E30" s="29"/>
     </row>
     <row r="31" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
@@ -4551,7 +4458,7 @@
       <c r="D31" s="6">
         <v>-1</v>
       </c>
-      <c r="E31" s="27"/>
+      <c r="E31" s="30"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
@@ -4566,7 +4473,7 @@
       <c r="D32" s="8">
         <v>1</v>
       </c>
-      <c r="E32" s="26" t="s">
+      <c r="E32" s="28" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4583,11 +4490,11 @@
       <c r="D33" s="2">
         <v>0</v>
       </c>
-      <c r="E33" s="30"/>
+      <c r="E33" s="29"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B34" s="2">
         <v>2</v>
@@ -4598,7 +4505,7 @@
       <c r="D34" s="2">
         <v>0</v>
       </c>
-      <c r="E34" s="30"/>
+      <c r="E34" s="29"/>
     </row>
     <row r="35" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
@@ -4613,7 +4520,7 @@
       <c r="D35" s="6">
         <v>-1</v>
       </c>
-      <c r="E35" s="27"/>
+      <c r="E35" s="30"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
@@ -4628,7 +4535,7 @@
       <c r="D36" s="8">
         <v>1</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="E36" s="28" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4645,7 +4552,7 @@
       <c r="D37" s="11">
         <v>-1</v>
       </c>
-      <c r="E37" s="27"/>
+      <c r="E37" s="30"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
@@ -4660,7 +4567,7 @@
       <c r="D38" s="8">
         <v>1</v>
       </c>
-      <c r="E38" s="26" t="s">
+      <c r="E38" s="28" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4677,7 +4584,7 @@
       <c r="D39" s="11">
         <v>-1</v>
       </c>
-      <c r="E39" s="27"/>
+      <c r="E39" s="30"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
@@ -4692,7 +4599,7 @@
       <c r="D40" s="8">
         <v>1</v>
       </c>
-      <c r="E40" s="26" t="s">
+      <c r="E40" s="28" t="s">
         <v>77</v>
       </c>
     </row>
@@ -4709,7 +4616,7 @@
       <c r="D41" s="2">
         <v>0</v>
       </c>
-      <c r="E41" s="30"/>
+      <c r="E41" s="29"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
@@ -4724,7 +4631,7 @@
       <c r="D42" s="2">
         <v>0</v>
       </c>
-      <c r="E42" s="30"/>
+      <c r="E42" s="29"/>
     </row>
     <row r="43" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
@@ -4739,7 +4646,7 @@
       <c r="D43" s="6">
         <v>-1</v>
       </c>
-      <c r="E43" s="27"/>
+      <c r="E43" s="30"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
@@ -4754,7 +4661,7 @@
       <c r="D44" s="8">
         <v>1</v>
       </c>
-      <c r="E44" s="26" t="s">
+      <c r="E44" s="28" t="s">
         <v>78</v>
       </c>
     </row>
@@ -4771,7 +4678,7 @@
       <c r="D45" s="2">
         <v>0</v>
       </c>
-      <c r="E45" s="30"/>
+      <c r="E45" s="29"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
@@ -4786,7 +4693,7 @@
       <c r="D46" s="2">
         <v>0</v>
       </c>
-      <c r="E46" s="30"/>
+      <c r="E46" s="29"/>
     </row>
     <row r="47" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
@@ -4801,7 +4708,7 @@
       <c r="D47" s="6">
         <v>-1</v>
       </c>
-      <c r="E47" s="27"/>
+      <c r="E47" s="30"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
@@ -4816,7 +4723,7 @@
       <c r="D48" s="8">
         <v>1</v>
       </c>
-      <c r="E48" s="26" t="s">
+      <c r="E48" s="28" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4833,7 +4740,7 @@
       <c r="D49" s="2">
         <v>0</v>
       </c>
-      <c r="E49" s="30"/>
+      <c r="E49" s="29"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
@@ -4848,7 +4755,7 @@
       <c r="D50" s="2">
         <v>0</v>
       </c>
-      <c r="E50" s="30"/>
+      <c r="E50" s="29"/>
     </row>
     <row r="51" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
@@ -4863,7 +4770,7 @@
       <c r="D51" s="6">
         <v>-1</v>
       </c>
-      <c r="E51" s="27"/>
+      <c r="E51" s="30"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
@@ -4878,7 +4785,7 @@
       <c r="D52" s="8">
         <v>1</v>
       </c>
-      <c r="E52" s="26" t="s">
+      <c r="E52" s="28" t="s">
         <v>80</v>
       </c>
     </row>
@@ -4895,7 +4802,7 @@
       <c r="D53" s="2">
         <v>0</v>
       </c>
-      <c r="E53" s="30"/>
+      <c r="E53" s="29"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
@@ -4910,7 +4817,7 @@
       <c r="D54" s="2">
         <v>0</v>
       </c>
-      <c r="E54" s="30"/>
+      <c r="E54" s="29"/>
     </row>
     <row r="55" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="12" t="s">
@@ -4925,11 +4832,11 @@
       <c r="D55" s="6">
         <v>-1</v>
       </c>
-      <c r="E55" s="30"/>
+      <c r="E55" s="29"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B56" s="8">
         <v>0</v>
@@ -4940,13 +4847,13 @@
       <c r="D56" s="8">
         <v>1</v>
       </c>
-      <c r="E56" s="28" t="s">
-        <v>491</v>
+      <c r="E56" s="26" t="s">
+        <v>489</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="12" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B57" s="6">
         <v>1</v>
@@ -4957,11 +4864,11 @@
       <c r="D57" s="6">
         <v>-1</v>
       </c>
-      <c r="E57" s="29"/>
+      <c r="E57" s="27"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B58" s="8">
         <v>0</v>
@@ -4972,13 +4879,13 @@
       <c r="D58" s="8">
         <v>1</v>
       </c>
-      <c r="E58" s="26" t="s">
-        <v>492</v>
+      <c r="E58" s="28" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="B59" s="2">
         <v>1</v>
@@ -4989,11 +4896,11 @@
       <c r="D59" s="2">
         <v>0</v>
       </c>
-      <c r="E59" s="30"/>
+      <c r="E59" s="29"/>
     </row>
     <row r="60" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B60" s="11">
         <v>2</v>
@@ -5004,10 +4911,20 @@
       <c r="D60" s="11">
         <v>-1</v>
       </c>
-      <c r="E60" s="27"/>
+      <c r="E60" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="E52:E55"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E14:E16"/>
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="E19:E22"/>
     <mergeCell ref="E40:E43"/>
@@ -5016,16 +4933,6 @@
     <mergeCell ref="E23:E27"/>
     <mergeCell ref="E28:E31"/>
     <mergeCell ref="E32:E35"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="E58:E60"/>
-    <mergeCell ref="E52:E55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
@@ -5154,7 +5061,7 @@
         <v>25</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>91</v>
@@ -5214,7 +5121,7 @@
         <v>25</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>3</v>
@@ -5235,7 +5142,7 @@
         <v>104</v>
       </c>
       <c r="S3" s="14" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="T3" s="15" t="s">
         <v>112</v>
@@ -5274,7 +5181,7 @@
         <v>140</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>91</v>
@@ -5330,7 +5237,7 @@
         <v>25</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>3</v>
@@ -5390,7 +5297,7 @@
         <v>140</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>91</v>
@@ -5450,7 +5357,7 @@
         <v>25</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>3</v>
@@ -5492,387 +5399,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE083F72-6C0E-4564-830C-AF36FA19A4AA}">
-  <dimension ref="A1:AL3"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.5546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" style="17" customWidth="1"/>
-    <col min="6" max="6" width="27.33203125" style="17" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="17.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="77.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.33203125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.109375" style="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="14.6640625" style="1" customWidth="1"/>
-    <col min="33" max="33" width="21.6640625" style="1" customWidth="1"/>
-    <col min="34" max="34" width="12.109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="12" style="1" customWidth="1"/>
-    <col min="36" max="36" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="5.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.5546875" style="1" customWidth="1"/>
-    <col min="39" max="39" width="8.88671875" style="1" customWidth="1"/>
-    <col min="40" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:38" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="H1" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="J1" s="13" t="s">
-        <v>206</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>207</v>
-      </c>
-      <c r="L1" s="13" t="s">
-        <v>208</v>
-      </c>
-      <c r="M1" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="N1" s="13" t="s">
-        <v>210</v>
-      </c>
-      <c r="O1" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>213</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="S1" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="T1" s="13" t="s">
-        <v>216</v>
-      </c>
-      <c r="U1" s="13" t="s">
-        <v>217</v>
-      </c>
-      <c r="V1" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="W1" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="X1" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="Y1" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="Z1" s="13" t="s">
-        <v>222</v>
-      </c>
-      <c r="AA1" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="AB1" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="AC1" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="AD1" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="AE1" s="13" t="s">
-        <v>227</v>
-      </c>
-      <c r="AF1" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="AG1" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="AH1" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="AI1" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="AJ1" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="AK1" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="AL1" s="13" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>545</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>549</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>547</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>549</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>546</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>550</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>551</v>
-      </c>
-      <c r="J2" s="2">
-        <v>1</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>551</v>
-      </c>
-      <c r="L2" s="2">
-        <v>1</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>557</v>
-      </c>
-      <c r="O2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="P2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="S2" s="2">
-        <v>14.99</v>
-      </c>
-      <c r="T2" s="2">
-        <v>17.989999999999998</v>
-      </c>
-      <c r="U2" s="2">
-        <v>19.989999999999998</v>
-      </c>
-      <c r="V2" s="2">
-        <v>12.99</v>
-      </c>
-      <c r="W2" s="2">
-        <v>30</v>
-      </c>
-      <c r="X2" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y2" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="Z2" s="2">
-        <v>50</v>
-      </c>
-      <c r="AA2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="15" t="s">
-        <v>580</v>
-      </c>
-      <c r="AC2" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="AD2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF2" s="20"/>
-      <c r="AG2" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH2" s="21"/>
-      <c r="AI2" s="21"/>
-      <c r="AJ2" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK2" s="15"/>
-      <c r="AL2" s="15" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>552</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>556</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>554</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>556</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>553</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>554</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>261</v>
-      </c>
-      <c r="J3" s="2">
-        <v>1</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>261</v>
-      </c>
-      <c r="L3" s="2">
-        <v>1</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>555</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>557</v>
-      </c>
-      <c r="O3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="P3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="S3" s="2">
-        <v>12.99</v>
-      </c>
-      <c r="T3" s="2">
-        <v>15.99</v>
-      </c>
-      <c r="U3" s="2">
-        <v>19.989999999999998</v>
-      </c>
-      <c r="V3" s="2">
-        <v>13.99</v>
-      </c>
-      <c r="W3" s="2">
-        <v>50</v>
-      </c>
-      <c r="X3" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y3" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="Z3" s="2">
-        <v>15</v>
-      </c>
-      <c r="AA3" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="15" t="s">
-        <v>581</v>
-      </c>
-      <c r="AC3" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="AD3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF3" s="20"/>
-      <c r="AG3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH3" s="21"/>
-      <c r="AI3" s="21"/>
-      <c r="AJ3" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK3" s="15"/>
-      <c r="AL3" s="15" t="s">
-        <v>559</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{303FC3B1-B557-4227-BB56-3144CCBBF032}">
   <dimension ref="A1:AL12"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -6037,7 +5563,7 @@
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>61</v>
@@ -6046,19 +5572,19 @@
         <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="G2" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>262</v>
@@ -6073,7 +5599,7 @@
         <v>1</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="N2" s="15" t="s">
         <v>253</v>
@@ -6138,12 +5664,12 @@
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>61</v>
@@ -6152,19 +5678,19 @@
         <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>55</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="I3" s="15" t="s">
         <v>262</v>
@@ -6179,7 +5705,7 @@
         <v>1</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="N3" s="15" t="s">
         <v>253</v>
@@ -6244,7 +5770,7 @@
       </c>
       <c r="AK3" s="23"/>
       <c r="AL3" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.3">
@@ -6261,7 +5787,7 @@
         <v>239</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="F4" s="24" t="s">
         <v>243</v>
@@ -6328,7 +5854,7 @@
         <v>263</v>
       </c>
       <c r="AB4" s="15" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="AC4" s="15" t="s">
         <v>91</v>
@@ -6346,10 +5872,10 @@
         <v>91</v>
       </c>
       <c r="AH4" s="22" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="AI4" s="22" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="AJ4" s="15" t="s">
         <v>3</v>
@@ -6373,7 +5899,7 @@
         <v>240</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>244</v>
@@ -6440,7 +5966,7 @@
         <v>263</v>
       </c>
       <c r="AB5" s="15" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="AC5" s="15" t="s">
         <v>91</v>
@@ -6456,10 +5982,10 @@
         <v>91</v>
       </c>
       <c r="AH5" s="22" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="AI5" s="22" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="AJ5" s="15" t="s">
         <v>3</v>
@@ -6480,7 +6006,7 @@
         <v>29</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>57</v>
@@ -6550,7 +6076,7 @@
         <v>263</v>
       </c>
       <c r="AB6" s="15" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="AC6" s="15" t="s">
         <v>91</v>
@@ -6566,10 +6092,10 @@
         <v>91</v>
       </c>
       <c r="AH6" s="22" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="AI6" s="22" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="AJ6" s="15" t="s">
         <v>3</v>
@@ -6590,7 +6116,7 @@
         <v>29</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>57</v>
@@ -6660,7 +6186,7 @@
         <v>263</v>
       </c>
       <c r="AB7" s="15" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="AC7" s="15" t="s">
         <v>91</v>
@@ -6678,10 +6204,10 @@
         <v>91</v>
       </c>
       <c r="AH7" s="22" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="AI7" s="22" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="AJ7" s="15" t="s">
         <v>3</v>
@@ -6696,7 +6222,7 @@
         <v>238</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>29</v>
@@ -6705,7 +6231,7 @@
         <v>241</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="F8" s="19" t="s">
         <v>247</v>
@@ -6772,7 +6298,7 @@
         <v>263</v>
       </c>
       <c r="AB8" s="15" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>91</v>
@@ -6799,28 +6325,28 @@
     </row>
     <row r="9" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>262</v>
@@ -6835,7 +6361,7 @@
         <v>1</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="N9" s="15" t="s">
         <v>253</v>
@@ -6878,7 +6404,7 @@
         <v>263</v>
       </c>
       <c r="AB9" s="15" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="AC9" s="19" t="s">
         <v>3</v>
@@ -6900,33 +6426,33 @@
       </c>
       <c r="AK9" s="2"/>
       <c r="AL9" s="2" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>261</v>
@@ -6941,7 +6467,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="N10" s="15" t="s">
         <v>253</v>
@@ -6984,7 +6510,7 @@
         <v>263</v>
       </c>
       <c r="AB10" s="15" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="AC10" s="19" t="s">
         <v>3</v>
@@ -7006,51 +6532,51 @@
       </c>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="E11" s="15" t="s">
         <v>547</v>
       </c>
-      <c r="E11" s="15" t="s">
-        <v>549</v>
-      </c>
       <c r="F11" s="15" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="J11" s="2">
         <v>1</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="L11" s="2">
         <v>1</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="O11" s="19" t="s">
         <v>3</v>
@@ -7090,7 +6616,7 @@
         <v>0</v>
       </c>
       <c r="AB11" s="15" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="AC11" s="15" t="s">
         <v>91</v>
@@ -7112,33 +6638,33 @@
       </c>
       <c r="AK11" s="15"/>
       <c r="AL11" s="15" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
     </row>
     <row r="12" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="E12" s="15" t="s">
         <v>554</v>
       </c>
-      <c r="E12" s="15" t="s">
-        <v>556</v>
-      </c>
       <c r="F12" s="15" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>261</v>
@@ -7153,10 +6679,10 @@
         <v>1</v>
       </c>
       <c r="M12" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>555</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>557</v>
       </c>
       <c r="O12" s="19" t="s">
         <v>3</v>
@@ -7196,7 +6722,7 @@
         <v>0</v>
       </c>
       <c r="AB12" s="15" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="AC12" s="15" t="s">
         <v>91</v>
@@ -7218,7 +6744,7 @@
       </c>
       <c r="AK12" s="15"/>
       <c r="AL12" s="15" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
   </sheetData>
@@ -7227,7 +6753,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F147CD6B-CA39-477C-82FD-5D86870A8EFB}">
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -7236,7 +6762,7 @@
     <col min="2" max="2" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" style="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" style="17" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" style="17" customWidth="1"/>
     <col min="7" max="7" width="38" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8.88671875" style="1"/>
@@ -7250,7 +6776,7 @@
         <v>126</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D1" s="13" t="s">
         <v>141</v>
@@ -7259,7 +6785,7 @@
         <v>231</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>209</v>
@@ -7267,10 +6793,10 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C2" s="19">
         <v>30</v>
@@ -7279,21 +6805,21 @@
         <v>29</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>282</v>
+        <v>542</v>
       </c>
       <c r="F2" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>290</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C3" s="1">
         <v>10</v>
@@ -7302,44 +6828,44 @@
         <v>29</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>295</v>
+        <v>542</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>287</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>288</v>
       </c>
       <c r="C4" s="19">
         <v>20</v>
       </c>
       <c r="D4" s="20" t="s">
+        <v>288</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>542</v>
+      </c>
+      <c r="F4" s="19" t="s">
         <v>289</v>
       </c>
-      <c r="E4" s="20" t="s">
-        <v>282</v>
-      </c>
-      <c r="F4" s="19" t="s">
-        <v>290</v>
-      </c>
       <c r="G4" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C5" s="19">
         <v>5</v>
@@ -7348,21 +6874,21 @@
         <v>29</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>282</v>
+        <v>542</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C6" s="19">
         <v>50</v>
@@ -7371,21 +6897,21 @@
         <v>29</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>282</v>
+        <v>542</v>
       </c>
       <c r="F6" s="19" t="s">
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C7" s="19">
         <v>10</v>
@@ -7394,21 +6920,21 @@
         <v>29</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>282</v>
+        <v>542</v>
       </c>
       <c r="F7" s="19" t="s">
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C8" s="19">
         <v>100</v>
@@ -7417,21 +6943,21 @@
         <v>29</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>282</v>
+        <v>542</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C9" s="19">
         <v>100</v>
@@ -7440,13 +6966,13 @@
         <v>29</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>282</v>
+        <v>542</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -7456,7 +6982,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C6C325F-4A76-431C-998A-38D75363C07E}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -7501,10 +7027,10 @@
         <v>1001</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>29</v>
@@ -7525,7 +7051,7 @@
         <v>53</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>62</v>
@@ -7545,10 +7071,10 @@
         <v>1003</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>32</v>
@@ -7566,7 +7092,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C7655F-AC18-4255-9C9F-28DEDD520460}">
   <dimension ref="A1:W9"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -7597,10 +7123,10 @@
   <sheetData>
     <row r="1" spans="1:23" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>85</v>
@@ -7621,7 +7147,7 @@
         <v>90</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="J1" s="13" t="s">
         <v>97</v>
@@ -7630,48 +7156,48 @@
         <v>96</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="O1" s="13" t="s">
         <v>202</v>
       </c>
       <c r="P1" s="13" t="s">
+        <v>309</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>310</v>
+      </c>
+      <c r="R1" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>312</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>313</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>314</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="W1" s="13" t="s">
         <v>316</v>
-      </c>
-      <c r="V1" s="13" t="s">
-        <v>317</v>
-      </c>
-      <c r="W1" s="13" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>99</v>
@@ -7692,16 +7218,16 @@
         <v>90001</v>
       </c>
       <c r="I2" s="15" t="s">
+        <v>319</v>
+      </c>
+      <c r="J2" s="15" t="s">
         <v>321</v>
       </c>
-      <c r="J2" s="15" t="s">
-        <v>323</v>
-      </c>
       <c r="K2" s="15" t="s">
+        <v>320</v>
+      </c>
+      <c r="L2" s="15" t="s">
         <v>322</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>324</v>
       </c>
       <c r="M2" s="19" t="s">
         <v>29</v>
@@ -7716,33 +7242,33 @@
         <v>91</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="R2" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="S2" s="15" t="s">
+        <v>324</v>
+      </c>
+      <c r="T2" s="15" t="s">
         <v>325</v>
-      </c>
-      <c r="S2" s="15" t="s">
-        <v>326</v>
-      </c>
-      <c r="T2" s="15" t="s">
-        <v>327</v>
       </c>
       <c r="U2" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="W2" s="19" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>114</v>
@@ -7763,16 +7289,16 @@
         <v>78701</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="M3" s="19" t="s">
         <v>29</v>
@@ -7787,33 +7313,33 @@
         <v>91</v>
       </c>
       <c r="Q3" s="19" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="R3" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="S3" s="15" t="s">
+        <v>331</v>
+      </c>
+      <c r="T3" s="15" t="s">
         <v>325</v>
-      </c>
-      <c r="S3" s="15" t="s">
-        <v>333</v>
-      </c>
-      <c r="T3" s="15" t="s">
-        <v>327</v>
       </c>
       <c r="U3" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V3" s="15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="W3" s="19" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>121</v>
@@ -7832,16 +7358,16 @@
         <v>75201</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="M4" s="19" t="s">
         <v>62</v>
@@ -7856,33 +7382,33 @@
         <v>91</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="R4" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="S4" s="15" t="s">
+        <v>332</v>
+      </c>
+      <c r="T4" s="15" t="s">
         <v>325</v>
-      </c>
-      <c r="S4" s="15" t="s">
-        <v>334</v>
-      </c>
-      <c r="T4" s="15" t="s">
-        <v>327</v>
       </c>
       <c r="U4" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="W4" s="19" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>128</v>
@@ -7903,22 +7429,22 @@
         <v>10118</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="M5" s="19" t="s">
         <v>29</v>
       </c>
       <c r="N5" s="19" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="O5" s="15" t="s">
         <v>47</v>
@@ -7927,33 +7453,33 @@
         <v>91</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="R5" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="S5" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="T5" s="15" t="s">
         <v>325</v>
-      </c>
-      <c r="S5" s="15" t="s">
-        <v>335</v>
-      </c>
-      <c r="T5" s="15" t="s">
-        <v>327</v>
       </c>
       <c r="U5" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="W5" s="19" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>135</v>
@@ -7974,16 +7500,16 @@
         <v>60606</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="M6" s="19" t="s">
         <v>29</v>
@@ -7998,33 +7524,33 @@
         <v>3</v>
       </c>
       <c r="Q6" s="19" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="R6" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="S6" s="15" t="s">
+        <v>334</v>
+      </c>
+      <c r="T6" s="15" t="s">
         <v>325</v>
-      </c>
-      <c r="S6" s="15" t="s">
-        <v>336</v>
-      </c>
-      <c r="T6" s="15" t="s">
-        <v>327</v>
       </c>
       <c r="U6" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="W6" s="19" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>135</v>
@@ -8045,22 +7571,22 @@
         <v>60606</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="M7" s="19" t="s">
         <v>29</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="O7" s="15" t="s">
         <v>47</v>
@@ -8069,25 +7595,25 @@
         <v>3</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="R7" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="S7" s="15" t="s">
+        <v>572</v>
+      </c>
+      <c r="T7" s="15" t="s">
         <v>325</v>
-      </c>
-      <c r="S7" s="15" t="s">
-        <v>574</v>
-      </c>
-      <c r="T7" s="15" t="s">
-        <v>327</v>
       </c>
       <c r="U7" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V7" s="15" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="W7" s="19" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.3">
@@ -8127,7 +7653,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3846B3E9-78EC-4A21-B7B1-295C9A6CBED2}">
   <dimension ref="A1:V5"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -8155,7 +7681,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>209</v>
@@ -8164,81 +7690,81 @@
         <v>126</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>351</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>352</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>353</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>354</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="H1" s="13" t="s">
         <v>355</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="I1" s="13" t="s">
         <v>356</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>357</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>358</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>359</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>360</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>361</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="O1" s="13" t="s">
         <v>362</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="P1" s="13" t="s">
         <v>363</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="Q1" s="13" t="s">
         <v>364</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>365</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>366</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>367</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>368</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>369</v>
-      </c>
-      <c r="U1" s="13" t="s">
-        <v>370</v>
-      </c>
-      <c r="V1" s="13" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>140</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="G2" s="2">
         <v>23.7044</v>
@@ -8292,13 +7818,13 @@
         <v>90</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>140</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="15"/>
@@ -8360,4 +7886,90 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5DA318D-8073-4D46-A062-C668992104C1}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>391</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>390</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>376</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>378</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>379</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>383</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>566</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>387</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
vehicle page element updated
</commit_message>
<xml_diff>
--- a/src/main/resources/ClientPortal_Data.xlsx
+++ b/src/main/resources/ClientPortal_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BS01361\My Folder\0. Test Type\4. Automation Testing\Selenium Files\MAS_FloraFire\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6849DCC1-2DD1-45D3-863C-7DD1975D54C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACAB312A-A55C-4620-A6B6-9872B86BC8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" tabRatio="803" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" tabRatio="803" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Value" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1225" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="586">
   <si>
     <t>Name</t>
   </si>
@@ -627,9 +627,6 @@
     <t>01/30/2024</t>
   </si>
   <si>
-    <t>06/30/2025</t>
-  </si>
-  <si>
     <t>11/15/2025</t>
   </si>
   <si>
@@ -1780,6 +1777,27 @@
   </si>
   <si>
     <t>5</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t>002</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>004</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t>Mileage</t>
   </si>
 </sst>
 </file>
@@ -2156,19 +2174,19 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2613,7 +2631,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B20" s="2">
         <v>18</v>
@@ -2621,7 +2639,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B21" s="2">
         <v>19</v>
@@ -2649,62 +2667,62 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>375</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>376</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>377</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>378</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>379</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D2" s="15" t="s">
+        <v>382</v>
+      </c>
+      <c r="E2" s="15" t="s">
         <v>383</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="F2" s="15" t="s">
         <v>384</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D3" s="15" t="s">
+        <v>385</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>383</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>386</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>384</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -2726,26 +2744,26 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>496</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -2777,310 +2795,310 @@
   <sheetData>
     <row r="1" spans="1:14" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>391</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>392</v>
       </c>
-      <c r="B1" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>393</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>394</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>395</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>396</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="H1" s="13" t="s">
+        <v>396</v>
+      </c>
+      <c r="I1" s="13" t="s">
         <v>397</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>398</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>399</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>400</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>401</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>402</v>
-      </c>
-      <c r="N1" s="13" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>410</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>411</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L2" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>412</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>91</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>91</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>91</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -3122,7 +3140,7 @@
         <v>144</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>85</v>
@@ -3146,27 +3164,27 @@
         <v>97</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="K1" s="13" t="s">
+        <v>468</v>
+      </c>
+      <c r="L1" s="13" t="s">
         <v>469</v>
-      </c>
-      <c r="L1" s="13" t="s">
-        <v>470</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>21</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>99</v>
@@ -3187,16 +3205,16 @@
         <v>90001</v>
       </c>
       <c r="I2" s="15" t="s">
+        <v>481</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>482</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>483</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>3</v>
@@ -3207,10 +3225,10 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>114</v>
@@ -3231,10 +3249,10 @@
         <v>78701</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>45</v>
@@ -3251,10 +3269,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>121</v>
@@ -3273,16 +3291,16 @@
         <v>75201</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>3</v>
@@ -3293,10 +3311,10 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>128</v>
@@ -3317,10 +3335,10 @@
         <v>10118</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>45</v>
@@ -3337,10 +3355,10 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>135</v>
@@ -3361,16 +3379,16 @@
         <v>60606</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>45</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>91</v>
@@ -3395,181 +3413,226 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE96B074-BAA6-41E4-A885-01589CFEB352}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="24.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="23.88671875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" style="1"/>
-    <col min="6" max="6" width="17.88671875" style="17" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" style="17" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="13.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.88671875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="17.88671875" style="17" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" style="17" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
+        <v>585</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="H1" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="I1" s="13" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="s">
+        <v>579</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E2" s="2">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="15" t="s">
+        <v>581</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>558</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E3" s="2">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>582</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="2">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="H4" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="I4" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="G2" s="15" t="s">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>583</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E5" s="2">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="I5" s="15" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>559</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="E4" s="2" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
+        <v>580</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="E6" s="2">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="18" t="s">
-        <v>189</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="H6" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="E7" s="2">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="15" t="s">
-        <v>192</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>193</v>
-      </c>
-      <c r="G6" s="15" t="s">
+      <c r="H7" s="15" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="15" t="s">
+      <c r="I7" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="G7" s="15" t="s">
-        <v>199</v>
-      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
@@ -3727,7 +3790,7 @@
   <sheetData>
     <row r="1" spans="1:39" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>126</v>
@@ -3736,117 +3799,117 @@
         <v>141</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="E1" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>0</v>
       </c>
       <c r="G1" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="I1" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="H1" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="O1" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="P1" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="Q1" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="W1" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="W1" s="13" t="s">
+      <c r="X1" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="Y1" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="Y1" s="13" t="s">
+      <c r="Z1" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="Z1" s="13" t="s">
+      <c r="AA1" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="AA1" s="13" t="s">
+      <c r="AB1" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="AB1" s="13" t="s">
+      <c r="AC1" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="AC1" s="13" t="s">
+      <c r="AD1" s="13" t="s">
         <v>225</v>
       </c>
-      <c r="AD1" s="13" t="s">
+      <c r="AE1" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="AE1" s="13" t="s">
+      <c r="AF1" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="AF1" s="13" t="s">
+      <c r="AG1" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="AG1" s="13" t="s">
+      <c r="AH1" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="AH1" s="13" t="s">
+      <c r="AI1" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="AI1" s="13" t="s">
+      <c r="AJ1" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="AJ1" s="13" t="s">
+      <c r="AK1" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="AK1" s="13" t="s">
-        <v>233</v>
-      </c>
       <c r="AL1" s="13" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="AM1" s="13" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>60</v>
@@ -3855,37 +3918,37 @@
         <v>29</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>58</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G2" s="23" t="s">
         <v>55</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J2" s="23">
         <v>70</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L2" s="23">
         <v>90</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O2" s="19" t="s">
         <v>3</v>
@@ -3947,7 +4010,7 @@
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="23" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="AM2" s="23" t="s">
         <v>91</v>
@@ -4002,7 +4065,7 @@
       <c r="D2" s="8">
         <v>1</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="28" t="s">
         <v>81</v>
       </c>
     </row>
@@ -4019,7 +4082,7 @@
       <c r="D3" s="2">
         <v>0</v>
       </c>
-      <c r="E3" s="30"/>
+      <c r="E3" s="29"/>
     </row>
     <row r="4" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
@@ -4034,7 +4097,7 @@
       <c r="D4" s="11">
         <v>-1</v>
       </c>
-      <c r="E4" s="27"/>
+      <c r="E4" s="30"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -4049,7 +4112,7 @@
       <c r="D5" s="8">
         <v>1</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="E5" s="28" t="s">
         <v>82</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -4069,7 +4132,7 @@
       <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
@@ -4084,7 +4147,7 @@
       <c r="D7" s="6">
         <v>-1</v>
       </c>
-      <c r="E7" s="27"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -4099,7 +4162,7 @@
       <c r="D8" s="8">
         <v>1</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="28" t="s">
         <v>83</v>
       </c>
     </row>
@@ -4116,7 +4179,7 @@
       <c r="D9" s="2">
         <v>0</v>
       </c>
-      <c r="E9" s="30"/>
+      <c r="E9" s="29"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
@@ -4131,7 +4194,7 @@
       <c r="D10" s="2">
         <v>0</v>
       </c>
-      <c r="E10" s="30"/>
+      <c r="E10" s="29"/>
     </row>
     <row r="11" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="12" t="s">
@@ -4146,7 +4209,7 @@
       <c r="D11" s="6">
         <v>-1</v>
       </c>
-      <c r="E11" s="30"/>
+      <c r="E11" s="29"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -4161,7 +4224,7 @@
       <c r="D12" s="8">
         <v>1</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="28" t="s">
         <v>68</v>
       </c>
     </row>
@@ -4178,7 +4241,7 @@
       <c r="D13" s="11">
         <v>-1</v>
       </c>
-      <c r="E13" s="27"/>
+      <c r="E13" s="30"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
@@ -4193,7 +4256,7 @@
       <c r="D14" s="8">
         <v>1</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="28" t="s">
         <v>69</v>
       </c>
     </row>
@@ -4210,7 +4273,7 @@
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="E15" s="30"/>
+      <c r="E15" s="29"/>
     </row>
     <row r="16" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
@@ -4225,7 +4288,7 @@
       <c r="D16" s="6">
         <v>-1</v>
       </c>
-      <c r="E16" s="27"/>
+      <c r="E16" s="30"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
@@ -4240,7 +4303,7 @@
       <c r="D17" s="8">
         <v>1</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="28" t="s">
         <v>70</v>
       </c>
     </row>
@@ -4257,7 +4320,7 @@
       <c r="D18" s="11">
         <v>-1</v>
       </c>
-      <c r="E18" s="27"/>
+      <c r="E18" s="30"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
@@ -4272,7 +4335,7 @@
       <c r="D19" s="8">
         <v>1</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="28" t="s">
         <v>71</v>
       </c>
     </row>
@@ -4289,7 +4352,7 @@
       <c r="D20" s="2">
         <v>0</v>
       </c>
-      <c r="E20" s="30"/>
+      <c r="E20" s="29"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
@@ -4304,7 +4367,7 @@
       <c r="D21" s="2">
         <v>0</v>
       </c>
-      <c r="E21" s="30"/>
+      <c r="E21" s="29"/>
     </row>
     <row r="22" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
@@ -4319,7 +4382,7 @@
       <c r="D22" s="6">
         <v>-1</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="30"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
@@ -4334,7 +4397,7 @@
       <c r="D23" s="8">
         <v>1</v>
       </c>
-      <c r="E23" s="26" t="s">
+      <c r="E23" s="28" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4351,7 +4414,7 @@
       <c r="D24" s="2">
         <v>0</v>
       </c>
-      <c r="E24" s="30"/>
+      <c r="E24" s="29"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
@@ -4366,7 +4429,7 @@
       <c r="D25" s="2">
         <v>0</v>
       </c>
-      <c r="E25" s="30"/>
+      <c r="E25" s="29"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
@@ -4381,7 +4444,7 @@
       <c r="D26" s="2">
         <v>0</v>
       </c>
-      <c r="E26" s="30"/>
+      <c r="E26" s="29"/>
     </row>
     <row r="27" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
@@ -4396,7 +4459,7 @@
       <c r="D27" s="11">
         <v>-1</v>
       </c>
-      <c r="E27" s="27"/>
+      <c r="E27" s="30"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
@@ -4411,7 +4474,7 @@
       <c r="D28" s="8">
         <v>1</v>
       </c>
-      <c r="E28" s="26" t="s">
+      <c r="E28" s="28" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4428,7 +4491,7 @@
       <c r="D29" s="2">
         <v>0</v>
       </c>
-      <c r="E29" s="30"/>
+      <c r="E29" s="29"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
@@ -4443,7 +4506,7 @@
       <c r="D30" s="2">
         <v>0</v>
       </c>
-      <c r="E30" s="30"/>
+      <c r="E30" s="29"/>
     </row>
     <row r="31" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
@@ -4458,7 +4521,7 @@
       <c r="D31" s="6">
         <v>-1</v>
       </c>
-      <c r="E31" s="27"/>
+      <c r="E31" s="30"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
@@ -4473,7 +4536,7 @@
       <c r="D32" s="8">
         <v>1</v>
       </c>
-      <c r="E32" s="26" t="s">
+      <c r="E32" s="28" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4490,11 +4553,11 @@
       <c r="D33" s="2">
         <v>0</v>
       </c>
-      <c r="E33" s="30"/>
+      <c r="E33" s="29"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B34" s="2">
         <v>2</v>
@@ -4505,7 +4568,7 @@
       <c r="D34" s="2">
         <v>0</v>
       </c>
-      <c r="E34" s="30"/>
+      <c r="E34" s="29"/>
     </row>
     <row r="35" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
@@ -4520,7 +4583,7 @@
       <c r="D35" s="6">
         <v>-1</v>
       </c>
-      <c r="E35" s="27"/>
+      <c r="E35" s="30"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
@@ -4535,7 +4598,7 @@
       <c r="D36" s="8">
         <v>1</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="E36" s="28" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4552,7 +4615,7 @@
       <c r="D37" s="11">
         <v>-1</v>
       </c>
-      <c r="E37" s="27"/>
+      <c r="E37" s="30"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
@@ -4567,7 +4630,7 @@
       <c r="D38" s="8">
         <v>1</v>
       </c>
-      <c r="E38" s="26" t="s">
+      <c r="E38" s="28" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4584,7 +4647,7 @@
       <c r="D39" s="11">
         <v>-1</v>
       </c>
-      <c r="E39" s="27"/>
+      <c r="E39" s="30"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
@@ -4599,13 +4662,13 @@
       <c r="D40" s="8">
         <v>1</v>
       </c>
-      <c r="E40" s="26" t="s">
+      <c r="E40" s="28" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B41" s="2">
         <v>1</v>
@@ -4616,7 +4679,7 @@
       <c r="D41" s="2">
         <v>0</v>
       </c>
-      <c r="E41" s="30"/>
+      <c r="E41" s="29"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
@@ -4631,7 +4694,7 @@
       <c r="D42" s="2">
         <v>0</v>
       </c>
-      <c r="E42" s="30"/>
+      <c r="E42" s="29"/>
     </row>
     <row r="43" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
@@ -4646,7 +4709,7 @@
       <c r="D43" s="6">
         <v>-1</v>
       </c>
-      <c r="E43" s="27"/>
+      <c r="E43" s="30"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
@@ -4661,7 +4724,7 @@
       <c r="D44" s="8">
         <v>1</v>
       </c>
-      <c r="E44" s="26" t="s">
+      <c r="E44" s="28" t="s">
         <v>78</v>
       </c>
     </row>
@@ -4678,7 +4741,7 @@
       <c r="D45" s="2">
         <v>0</v>
       </c>
-      <c r="E45" s="30"/>
+      <c r="E45" s="29"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
@@ -4693,7 +4756,7 @@
       <c r="D46" s="2">
         <v>0</v>
       </c>
-      <c r="E46" s="30"/>
+      <c r="E46" s="29"/>
     </row>
     <row r="47" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
@@ -4708,7 +4771,7 @@
       <c r="D47" s="6">
         <v>-1</v>
       </c>
-      <c r="E47" s="27"/>
+      <c r="E47" s="30"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
@@ -4723,7 +4786,7 @@
       <c r="D48" s="8">
         <v>1</v>
       </c>
-      <c r="E48" s="26" t="s">
+      <c r="E48" s="28" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4740,7 +4803,7 @@
       <c r="D49" s="2">
         <v>0</v>
       </c>
-      <c r="E49" s="30"/>
+      <c r="E49" s="29"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
@@ -4755,7 +4818,7 @@
       <c r="D50" s="2">
         <v>0</v>
       </c>
-      <c r="E50" s="30"/>
+      <c r="E50" s="29"/>
     </row>
     <row r="51" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
@@ -4770,7 +4833,7 @@
       <c r="D51" s="6">
         <v>-1</v>
       </c>
-      <c r="E51" s="27"/>
+      <c r="E51" s="30"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
@@ -4785,7 +4848,7 @@
       <c r="D52" s="8">
         <v>1</v>
       </c>
-      <c r="E52" s="26" t="s">
+      <c r="E52" s="28" t="s">
         <v>80</v>
       </c>
     </row>
@@ -4802,7 +4865,7 @@
       <c r="D53" s="2">
         <v>0</v>
       </c>
-      <c r="E53" s="30"/>
+      <c r="E53" s="29"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
@@ -4817,7 +4880,7 @@
       <c r="D54" s="2">
         <v>0</v>
       </c>
-      <c r="E54" s="30"/>
+      <c r="E54" s="29"/>
     </row>
     <row r="55" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="12" t="s">
@@ -4832,11 +4895,11 @@
       <c r="D55" s="6">
         <v>-1</v>
       </c>
-      <c r="E55" s="30"/>
+      <c r="E55" s="29"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B56" s="8">
         <v>0</v>
@@ -4847,13 +4910,13 @@
       <c r="D56" s="8">
         <v>1</v>
       </c>
-      <c r="E56" s="28" t="s">
-        <v>489</v>
+      <c r="E56" s="26" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B57" s="6">
         <v>1</v>
@@ -4864,11 +4927,11 @@
       <c r="D57" s="6">
         <v>-1</v>
       </c>
-      <c r="E57" s="29"/>
+      <c r="E57" s="27"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B58" s="8">
         <v>0</v>
@@ -4879,13 +4942,13 @@
       <c r="D58" s="8">
         <v>1</v>
       </c>
-      <c r="E58" s="26" t="s">
-        <v>490</v>
+      <c r="E58" s="28" t="s">
+        <v>489</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B59" s="2">
         <v>1</v>
@@ -4896,11 +4959,11 @@
       <c r="D59" s="2">
         <v>0</v>
       </c>
-      <c r="E59" s="30"/>
+      <c r="E59" s="29"/>
     </row>
     <row r="60" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B60" s="11">
         <v>2</v>
@@ -4911,10 +4974,20 @@
       <c r="D60" s="11">
         <v>-1</v>
       </c>
-      <c r="E60" s="27"/>
+      <c r="E60" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="E52:E55"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E14:E16"/>
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="E19:E22"/>
     <mergeCell ref="E40:E43"/>
@@ -4923,16 +4996,6 @@
     <mergeCell ref="E23:E27"/>
     <mergeCell ref="E28:E31"/>
     <mergeCell ref="E32:E35"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="E58:E60"/>
-    <mergeCell ref="E52:E55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
@@ -5061,7 +5124,7 @@
         <v>25</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>91</v>
@@ -5121,7 +5184,7 @@
         <v>25</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>3</v>
@@ -5142,7 +5205,7 @@
         <v>104</v>
       </c>
       <c r="S3" s="14" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="T3" s="15" t="s">
         <v>112</v>
@@ -5181,7 +5244,7 @@
         <v>140</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>91</v>
@@ -5237,7 +5300,7 @@
         <v>25</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>3</v>
@@ -5297,7 +5360,7 @@
         <v>140</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>91</v>
@@ -5357,7 +5420,7 @@
         <v>25</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>3</v>
@@ -5447,7 +5510,7 @@
   <sheetData>
     <row r="1" spans="1:38" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>126</v>
@@ -5456,114 +5519,114 @@
         <v>141</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="E1" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>0</v>
       </c>
       <c r="G1" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="I1" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="H1" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="O1" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="P1" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="Q1" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="W1" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="W1" s="13" t="s">
+      <c r="X1" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="Y1" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="Y1" s="13" t="s">
+      <c r="Z1" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="Z1" s="13" t="s">
+      <c r="AA1" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="AA1" s="13" t="s">
+      <c r="AB1" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="AB1" s="13" t="s">
+      <c r="AC1" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="AC1" s="13" t="s">
+      <c r="AD1" s="13" t="s">
         <v>225</v>
       </c>
-      <c r="AD1" s="13" t="s">
+      <c r="AE1" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="AE1" s="13" t="s">
+      <c r="AF1" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="AF1" s="13" t="s">
+      <c r="AG1" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="AG1" s="13" t="s">
+      <c r="AH1" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="AH1" s="13" t="s">
+      <c r="AI1" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="AI1" s="13" t="s">
+      <c r="AJ1" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="AJ1" s="13" t="s">
+      <c r="AK1" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="AK1" s="13" t="s">
-        <v>233</v>
-      </c>
       <c r="AL1" s="13" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>61</v>
@@ -5572,37 +5635,37 @@
         <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="G2" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J2" s="2">
         <v>1</v>
       </c>
       <c r="K2" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L2" s="2">
         <v>1</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O2" s="15" t="s">
         <v>91</v>
@@ -5664,12 +5727,12 @@
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>61</v>
@@ -5678,37 +5741,37 @@
         <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>61</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>55</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J3" s="2">
         <v>1</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L3" s="2">
         <v>1</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="N3" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O3" s="19" t="s">
         <v>3</v>
@@ -5770,12 +5833,12 @@
       </c>
       <c r="AK3" s="23"/>
       <c r="AL3" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B4" s="19" t="s">
         <v>60</v>
@@ -5784,37 +5847,37 @@
         <v>29</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G4" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="N4" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O4" s="19" t="s">
         <v>3</v>
@@ -5836,7 +5899,7 @@
         <v>9.99</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="W4" s="19">
         <v>5.99</v>
@@ -5851,10 +5914,10 @@
         <v>100</v>
       </c>
       <c r="AA4" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AB4" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AC4" s="15" t="s">
         <v>91</v>
@@ -5866,28 +5929,28 @@
         <v>91</v>
       </c>
       <c r="AF4" s="20" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="AG4" s="15" t="s">
         <v>91</v>
       </c>
       <c r="AH4" s="22" t="s">
+        <v>540</v>
+      </c>
+      <c r="AI4" s="22" t="s">
         <v>541</v>
-      </c>
-      <c r="AI4" s="22" t="s">
-        <v>542</v>
       </c>
       <c r="AJ4" s="15" t="s">
         <v>3</v>
       </c>
       <c r="AK4" s="15"/>
       <c r="AL4" s="15" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>60</v>
@@ -5896,37 +5959,37 @@
         <v>62</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G5" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O5" s="15" t="s">
         <v>91</v>
@@ -5948,7 +6011,7 @@
         <v>25.99</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="W5" s="19">
         <v>15.99</v>
@@ -5963,10 +6026,10 @@
         <v>75</v>
       </c>
       <c r="AA5" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AB5" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AC5" s="15" t="s">
         <v>91</v>
@@ -5982,22 +6045,22 @@
         <v>91</v>
       </c>
       <c r="AH5" s="22" t="s">
+        <v>540</v>
+      </c>
+      <c r="AI5" s="22" t="s">
         <v>541</v>
-      </c>
-      <c r="AI5" s="22" t="s">
-        <v>542</v>
       </c>
       <c r="AJ5" s="15" t="s">
         <v>3</v>
       </c>
       <c r="AK5" s="15"/>
       <c r="AL5" s="15" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>57</v>
@@ -6006,37 +6069,37 @@
         <v>29</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>57</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G6" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="M6" s="19" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O6" s="15" t="s">
         <v>91</v>
@@ -6058,7 +6121,7 @@
         <v>59.99</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="W6" s="19">
         <v>39.99</v>
@@ -6073,10 +6136,10 @@
         <v>30</v>
       </c>
       <c r="AA6" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AB6" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AC6" s="15" t="s">
         <v>91</v>
@@ -6092,22 +6155,22 @@
         <v>91</v>
       </c>
       <c r="AH6" s="22" t="s">
+        <v>540</v>
+      </c>
+      <c r="AI6" s="22" t="s">
         <v>541</v>
-      </c>
-      <c r="AI6" s="22" t="s">
-        <v>542</v>
       </c>
       <c r="AJ6" s="15" t="s">
         <v>3</v>
       </c>
       <c r="AK6" s="15"/>
       <c r="AL6" s="15" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>57</v>
@@ -6116,37 +6179,37 @@
         <v>29</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>57</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O7" s="15" t="s">
         <v>91</v>
@@ -6168,7 +6231,7 @@
         <v>45.99</v>
       </c>
       <c r="V7" s="15" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="W7" s="19">
         <v>25.99</v>
@@ -6183,10 +6246,10 @@
         <v>60</v>
       </c>
       <c r="AA7" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AB7" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AC7" s="15" t="s">
         <v>91</v>
@@ -6198,67 +6261,67 @@
         <v>91</v>
       </c>
       <c r="AF7" s="20" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="AG7" s="15" t="s">
         <v>91</v>
       </c>
       <c r="AH7" s="22" t="s">
+        <v>540</v>
+      </c>
+      <c r="AI7" s="22" t="s">
         <v>541</v>
-      </c>
-      <c r="AI7" s="22" t="s">
-        <v>542</v>
       </c>
       <c r="AJ7" s="15" t="s">
         <v>3</v>
       </c>
       <c r="AK7" s="15"/>
       <c r="AL7" s="15" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L8" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="M8" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="N8" s="15" t="s">
         <v>252</v>
-      </c>
-      <c r="N8" s="15" t="s">
-        <v>253</v>
       </c>
       <c r="O8" s="15" t="s">
         <v>91</v>
@@ -6280,7 +6343,7 @@
         <v>8.99</v>
       </c>
       <c r="V8" s="15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="W8" s="19">
         <v>4.99</v>
@@ -6295,10 +6358,10 @@
         <v>200</v>
       </c>
       <c r="AA8" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AB8" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AC8" s="15" t="s">
         <v>91</v>
@@ -6320,51 +6383,51 @@
       </c>
       <c r="AK8" s="15"/>
       <c r="AL8" s="15" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J9" s="2">
         <v>1</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L9" s="2">
         <v>1</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="N9" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O9" s="19" t="s">
         <v>3</v>
@@ -6401,10 +6464,10 @@
         <v>50</v>
       </c>
       <c r="AA9" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AB9" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AC9" s="19" t="s">
         <v>3</v>
@@ -6426,51 +6489,51 @@
       </c>
       <c r="AK9" s="2"/>
       <c r="AL9" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J10" s="2">
         <v>1</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L10" s="2">
         <v>1</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="N10" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O10" s="15" t="s">
         <v>91</v>
@@ -6507,10 +6570,10 @@
         <v>20</v>
       </c>
       <c r="AA10" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AB10" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AC10" s="19" t="s">
         <v>3</v>
@@ -6532,51 +6595,51 @@
       </c>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>55</v>
       </c>
       <c r="H11" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>548</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="J11" s="2">
         <v>1</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="L11" s="2">
         <v>1</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="O11" s="19" t="s">
         <v>3</v>
@@ -6616,7 +6679,7 @@
         <v>0</v>
       </c>
       <c r="AB11" s="15" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AC11" s="15" t="s">
         <v>91</v>
@@ -6638,51 +6701,51 @@
       </c>
       <c r="AK11" s="15"/>
       <c r="AL11" s="15" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="12" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>54</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J12" s="2">
         <v>1</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L12" s="2">
         <v>1</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="O12" s="19" t="s">
         <v>3</v>
@@ -6722,7 +6785,7 @@
         <v>0</v>
       </c>
       <c r="AB12" s="15" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AC12" s="15" t="s">
         <v>91</v>
@@ -6744,7 +6807,7 @@
       </c>
       <c r="AK12" s="15"/>
       <c r="AL12" s="15" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
   </sheetData>
@@ -6770,33 +6833,33 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>126</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C2" s="19">
         <v>30</v>
@@ -6805,21 +6868,21 @@
         <v>29</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F2" s="19" t="s">
+        <v>288</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C3" s="1">
         <v>10</v>
@@ -6828,44 +6891,44 @@
         <v>29</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
+        <v>285</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>286</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>287</v>
       </c>
       <c r="C4" s="19">
         <v>20</v>
       </c>
       <c r="D4" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>541</v>
+      </c>
+      <c r="F4" s="19" t="s">
         <v>288</v>
       </c>
-      <c r="E4" s="20" t="s">
-        <v>542</v>
-      </c>
-      <c r="F4" s="19" t="s">
-        <v>289</v>
-      </c>
       <c r="G4" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C5" s="19">
         <v>5</v>
@@ -6874,21 +6937,21 @@
         <v>29</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C6" s="19">
         <v>50</v>
@@ -6897,21 +6960,21 @@
         <v>29</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F6" s="19" t="s">
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C7" s="19">
         <v>10</v>
@@ -6920,21 +6983,21 @@
         <v>29</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F7" s="19" t="s">
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C8" s="19">
         <v>100</v>
@@ -6943,21 +7006,21 @@
         <v>29</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F8" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>300</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C9" s="19">
         <v>100</v>
@@ -6966,13 +7029,13 @@
         <v>29</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -7001,36 +7064,36 @@
         <v>126</v>
       </c>
       <c r="B1" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>276</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>277</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>278</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="F1" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="G1" s="13" t="s">
         <v>279</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B2" s="19">
         <v>1001</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>29</v>
@@ -7042,7 +7105,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B3" s="19">
         <v>1002</v>
@@ -7051,7 +7114,7 @@
         <v>53</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>62</v>
@@ -7065,16 +7128,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B4" s="19">
         <v>1003</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>32</v>
@@ -7123,10 +7186,10 @@
   <sheetData>
     <row r="1" spans="1:23" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>304</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>305</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>85</v>
@@ -7147,7 +7210,7 @@
         <v>90</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="J1" s="13" t="s">
         <v>97</v>
@@ -7156,48 +7219,48 @@
         <v>96</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>141</v>
       </c>
       <c r="N1" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="O1" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="P1" s="13" t="s">
         <v>308</v>
       </c>
-      <c r="O1" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="P1" s="13" t="s">
+      <c r="Q1" s="13" t="s">
         <v>309</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>312</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>313</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>314</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="W1" s="13" t="s">
         <v>315</v>
-      </c>
-      <c r="W1" s="13" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
+        <v>316</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>317</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>318</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>99</v>
@@ -7218,16 +7281,16 @@
         <v>90001</v>
       </c>
       <c r="I2" s="15" t="s">
+        <v>318</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>320</v>
+      </c>
+      <c r="K2" s="15" t="s">
         <v>319</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="L2" s="15" t="s">
         <v>321</v>
-      </c>
-      <c r="K2" s="15" t="s">
-        <v>320</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>322</v>
       </c>
       <c r="M2" s="19" t="s">
         <v>29</v>
@@ -7242,33 +7305,33 @@
         <v>91</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="R2" s="15" t="s">
+        <v>322</v>
+      </c>
+      <c r="S2" s="15" t="s">
         <v>323</v>
       </c>
-      <c r="S2" s="15" t="s">
+      <c r="T2" s="15" t="s">
         <v>324</v>
-      </c>
-      <c r="T2" s="15" t="s">
-        <v>325</v>
       </c>
       <c r="U2" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="W2" s="19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
+        <v>326</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>327</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>328</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>114</v>
@@ -7289,16 +7352,16 @@
         <v>78701</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="M3" s="19" t="s">
         <v>29</v>
@@ -7313,33 +7376,33 @@
         <v>91</v>
       </c>
       <c r="Q3" s="19" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="R3" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="S3" s="15" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="T3" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="U3" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V3" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="W3" s="19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>121</v>
@@ -7358,16 +7421,16 @@
         <v>75201</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="L4" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="M4" s="19" t="s">
         <v>62</v>
@@ -7382,33 +7445,33 @@
         <v>91</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="R4" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="S4" s="15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="T4" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="U4" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V4" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="W4" s="19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
+        <v>341</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>342</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>343</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>128</v>
@@ -7429,22 +7492,22 @@
         <v>10118</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="M5" s="19" t="s">
         <v>29</v>
       </c>
       <c r="N5" s="19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="O5" s="15" t="s">
         <v>47</v>
@@ -7453,33 +7516,33 @@
         <v>91</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R5" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="S5" s="15" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="T5" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="U5" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V5" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="W5" s="19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
+        <v>343</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>344</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>345</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>135</v>
@@ -7500,16 +7563,16 @@
         <v>60606</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="L6" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="M6" s="19" t="s">
         <v>29</v>
@@ -7524,33 +7587,33 @@
         <v>3</v>
       </c>
       <c r="Q6" s="19" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="R6" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="S6" s="15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="T6" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="U6" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V6" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="W6" s="19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>567</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>568</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>135</v>
@@ -7571,22 +7634,22 @@
         <v>60606</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="L7" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="M7" s="19" t="s">
         <v>29</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="O7" s="15" t="s">
         <v>47</v>
@@ -7595,25 +7658,25 @@
         <v>3</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="R7" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="S7" s="15" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="T7" s="15" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="U7" s="15" t="s">
         <v>127</v>
       </c>
       <c r="V7" s="15" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="W7" s="19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.3">
@@ -7681,90 +7744,90 @@
   <sheetData>
     <row r="1" spans="1:22" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>126</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>350</v>
+      </c>
+      <c r="E1" s="13" t="s">
         <v>351</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>352</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>353</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="H1" s="13" t="s">
         <v>354</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="I1" s="13" t="s">
         <v>355</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="13" t="s">
         <v>356</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="13" t="s">
         <v>357</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="13" t="s">
         <v>358</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="13" t="s">
         <v>359</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="13" t="s">
         <v>360</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="O1" s="13" t="s">
         <v>361</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="P1" s="13" t="s">
         <v>362</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="Q1" s="13" t="s">
         <v>363</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="R1" s="13" t="s">
         <v>364</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>365</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="T1" s="13" t="s">
         <v>366</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="U1" s="13" t="s">
         <v>367</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>368</v>
-      </c>
-      <c r="V1" s="13" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>370</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>371</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>140</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E2" s="15" t="s">
+        <v>372</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>373</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>374</v>
       </c>
       <c r="G2" s="2">
         <v>23.7044</v>
@@ -7818,13 +7881,13 @@
         <v>90</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>140</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="15"/>
@@ -7901,71 +7964,71 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C1" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="D1" s="13" t="s">
         <v>376</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="E1" s="13" t="s">
         <v>377</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="F1" s="13" t="s">
         <v>378</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="G1" s="13" t="s">
         <v>379</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>90</v>
       </c>
       <c r="E2" s="15" t="s">
+        <v>382</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>383</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="G2" s="15" t="s">
         <v>384</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>90</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>

</xml_diff>